<commit_message>
Update recruitment ratio workbook
</commit_message>
<xml_diff>
--- a/채용비율.xlsx
+++ b/채용비율.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1.26년 전체 소속별 점유율" sheetId="1" r:id="R3e1053f457d943fa"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2.각8개지부 현장점유율" sheetId="2" r:id="R3df2097710f24f3f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3.타워사별 점유현황" sheetId="3" r:id="R0e3bd4c6d0c840d5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4.반도체현장" sheetId="4" r:id="Rab0994875a9b4b60"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5.1~9월채용추이" sheetId="5" r:id="Rc725e3da583e4bda"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="6.월별 소속별 채용비율" sheetId="6" r:id="R3c5b08d230cb40d0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1.26년 전체 소속별 점유율" sheetId="1" r:id="Rf9a42abcac194542"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2.각8개지부 현장점유율" sheetId="2" r:id="R575daa7d0bb2459a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3.타워사별 점유현황" sheetId="3" r:id="R51d5626cf6584477"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4.반도체현장" sheetId="4" r:id="R375fd11df0e240ae"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5.1~9월채용추이" sheetId="5" r:id="Ra1f275c8a34d4eab"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="6.월별 소속별 채용비율" sheetId="6" r:id="R118a5c739999476d"/>
   </x:sheets>
   <x:definedNames>
     <x:definedName name="가평군">#REF!</x:definedName>
@@ -381,9 +381,6 @@
   </x:si>
   <x:si>
     <x:t xml:space="preserve">p4 복합동(배정완료)</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">기흥 NRD K2</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">민주식 010-4870-9982</x:t>
@@ -3417,7 +3414,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rf9e9f69380ed4c77"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R0991f3956ad24826"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -8424,15 +8421,15 @@
     <x:row r="6">
       <x:c r="A6" s="16" t="n">
         <x:f t="shared" ref="A6:F6" si="0">SUM(C11:C20)</x:f>
-        <x:v>132</x:v>
+        <x:v>138</x:v>
       </x:c>
       <x:c r="B6" s="16" t="n">
         <x:f t="shared" si="0"/>
-        <x:v>48</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="C6" s="16" t="n">
         <x:f t="shared" si="0"/>
-        <x:v>57</x:v>
+        <x:v>59</x:v>
       </x:c>
       <x:c r="D6" s="16" t="n">
         <x:f t="shared" si="0"/>
@@ -8444,7 +8441,7 @@
       </x:c>
       <x:c r="F6" s="16" t="n">
         <x:f t="shared" si="0"/>
-        <x:v>13</x:v>
+        <x:v>16</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -8452,19 +8449,19 @@
         <x:v>96</x:v>
       </x:c>
       <x:c r="B7" s="35" t="n">
-        <x:v>0.36363636363636365</x:v>
+        <x:v>0.35507246376811596</x:v>
       </x:c>
       <x:c r="C7" s="35" t="n">
-        <x:v>0.4318181818181818</x:v>
+        <x:v>0.427536231884058</x:v>
       </x:c>
       <x:c r="D7" s="35" t="n">
-        <x:v>0.015151515151515152</x:v>
+        <x:v>0.014492753623188406</x:v>
       </x:c>
       <x:c r="E7" s="35" t="n">
-        <x:v>0.09090909090909091</x:v>
+        <x:v>0.08695652173913043</x:v>
       </x:c>
       <x:c r="F7" s="35" t="n">
-        <x:v>0.09848484848484848</x:v>
+        <x:v>0.11594202898550725</x:v>
       </x:c>
     </x:row>
     <x:row r="9" s="14" customFormat="1" ht="15.399999618530273" customHeight="1">
@@ -8658,29 +8655,29 @@
       <x:c r="A16" s="24">
         <x:v>6</x:v>
       </x:c>
-      <x:c r="B16" s="25" t="s">
+      <x:c r="B16" s="25" t="str">
+        <x:v>기흥 NRD FAB동</x:v>
+      </x:c>
+      <x:c r="C16" s="26" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="D16" s="27" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E16" s="27" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="F16" s="27" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G16" s="27" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H16" s="27" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I16" s="28" t="s">
         <x:v>111</x:v>
-      </x:c>
-      <x:c r="C16" s="26">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="D16" s="27">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="E16" s="27">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="F16" s="27">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G16" s="27">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="H16" s="27">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="I16" s="28" t="s">
-        <x:v>112</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
@@ -8688,7 +8685,7 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="B17" s="20" t="s">
-        <x:v>113</x:v>
+        <x:v>112</x:v>
       </x:c>
       <x:c r="C17" s="21">
         <x:v>15</x:v>
@@ -8709,7 +8706,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="I17" s="23" t="s">
-        <x:v>114</x:v>
+        <x:v>113</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
@@ -8717,7 +8714,7 @@
         <x:v>8</x:v>
       </x:c>
       <x:c r="B18" s="25" t="s">
-        <x:v>115</x:v>
+        <x:v>114</x:v>
       </x:c>
       <x:c r="C18" s="26">
         <x:v>5</x:v>
@@ -8738,7 +8735,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="I18" s="28" t="s">
-        <x:v>116</x:v>
+        <x:v>115</x:v>
       </x:c>
     </x:row>
     <x:row r="19">
@@ -8746,28 +8743,28 @@
         <x:v>9</x:v>
       </x:c>
       <x:c r="B19" s="20" t="s">
+        <x:v>116</x:v>
+      </x:c>
+      <x:c r="C19" s="21">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="D19" s="22">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E19" s="22">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F19" s="22">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G19" s="22">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H19" s="22">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I19" s="23" t="s">
         <x:v>117</x:v>
-      </x:c>
-      <x:c r="C19" s="21">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="D19" s="22">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E19" s="22">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="F19" s="22">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G19" s="22">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="H19" s="22">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="I19" s="23" t="s">
-        <x:v>118</x:v>
       </x:c>
     </x:row>
     <x:row r="20" s="14" customFormat="1" ht="14.449999809265137" customHeight="1">
@@ -8775,7 +8772,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="B20" s="25" t="s">
-        <x:v>119</x:v>
+        <x:v>118</x:v>
       </x:c>
       <x:c r="C20" s="26">
         <x:v>6</x:v>
@@ -8808,7 +8805,7 @@
       </x:c>
       <x:c r="C21" s="31" t="n">
         <x:f t="shared" ref="C21:H21" si="1">SUM(C11:C20)</x:f>
-        <x:v>2</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="D21" s="31" t="n">
         <x:f t="shared" si="1"/>
@@ -8816,7 +8813,7 @@
       </x:c>
       <x:c r="E21" s="31" t="n">
         <x:f t="shared" si="1"/>
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="F21" s="31" t="n">
         <x:f t="shared" si="1"/>
@@ -8828,7 +8825,7 @@
       </x:c>
       <x:c r="H21" s="31" t="n">
         <x:f t="shared" si="1"/>
-        <x:v>0</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="I21" s="29" t="str">
         <x:v>신규 현장 · 신우개발(주) / 삼성이앤에이(주)</x:v>
@@ -8840,13 +8837,13 @@
         <x:v>합 계</x:v>
       </x:c>
       <x:c r="C22" t="n">
-        <x:v>132</x:v>
+        <x:v>138</x:v>
       </x:c>
       <x:c r="D22" t="n">
-        <x:v>48</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="E22" t="n">
-        <x:v>57</x:v>
+        <x:v>59</x:v>
       </x:c>
       <x:c r="F22" t="n">
         <x:v>2</x:v>
@@ -8855,7 +8852,7 @@
         <x:v>12</x:v>
       </x:c>
       <x:c r="H22" t="n">
-        <x:v>13</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="I22"/>
     </x:row>
@@ -8886,7 +8883,7 @@
   <x:sheetData>
     <x:row r="1" s="14" customFormat="1" ht="15.399999618530273" customHeight="1">
       <x:c r="A1" s="192" t="s">
-        <x:v>120</x:v>
+        <x:v>119</x:v>
       </x:c>
       <x:c r="B1" s="193"/>
       <x:c r="C1" s="193"/>
@@ -8900,10 +8897,10 @@
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="40" t="s">
+        <x:v>120</x:v>
+      </x:c>
+      <x:c r="B2" s="40" t="s">
         <x:v>121</x:v>
-      </x:c>
-      <x:c r="B2" s="40" t="s">
-        <x:v>122</x:v>
       </x:c>
       <x:c r="C2" s="40" t="s">
         <x:v>14</x:v>
@@ -8918,7 +8915,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G2" s="40" t="s">
-        <x:v>123</x:v>
+        <x:v>122</x:v>
       </x:c>
       <x:c r="H2" s="40" t="s">
         <x:v>6</x:v>
@@ -8947,10 +8944,10 @@
         <x:v>31</x:v>
       </x:c>
       <x:c r="B4" s="41" t="s">
+        <x:v>123</x:v>
+      </x:c>
+      <x:c r="C4" s="43" t="s">
         <x:v>124</x:v>
-      </x:c>
-      <x:c r="C4" s="43" t="s">
-        <x:v>125</x:v>
       </x:c>
       <x:c r="D4" s="42">
         <x:v>5</x:v>
@@ -9042,7 +9039,7 @@
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="194" t="s">
-        <x:v>126</x:v>
+        <x:v>125</x:v>
       </x:c>
       <x:c r="B9" s="193"/>
       <x:c r="C9" s="193"/>
@@ -9086,7 +9083,7 @@
     </x:row>
     <x:row r="11" s="14" customFormat="1" ht="15.399999618530273" customHeight="1">
       <x:c r="A11" s="192" t="s">
-        <x:v>127</x:v>
+        <x:v>126</x:v>
       </x:c>
       <x:c r="B11" s="193"/>
       <x:c r="C11" s="193"/>
@@ -9100,10 +9097,10 @@
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="40" t="s">
+        <x:v>120</x:v>
+      </x:c>
+      <x:c r="B12" s="40" t="s">
         <x:v>121</x:v>
-      </x:c>
-      <x:c r="B12" s="40" t="s">
-        <x:v>122</x:v>
       </x:c>
       <x:c r="C12" s="40" t="s">
         <x:v>14</x:v>
@@ -9118,7 +9115,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G12" s="40" t="s">
-        <x:v>123</x:v>
+        <x:v>122</x:v>
       </x:c>
       <x:c r="H12" s="40" t="s">
         <x:v>6</x:v>
@@ -9135,10 +9132,10 @@
         <x:v>65</x:v>
       </x:c>
       <x:c r="B13" s="41" t="s">
+        <x:v>127</x:v>
+      </x:c>
+      <x:c r="C13" s="43" t="s">
         <x:v>128</x:v>
-      </x:c>
-      <x:c r="C13" s="43" t="s">
-        <x:v>129</x:v>
       </x:c>
       <x:c r="D13" s="42">
         <x:v>4</x:v>
@@ -9165,10 +9162,10 @@
         <x:v>29</x:v>
       </x:c>
       <x:c r="B14" s="42" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="C14" s="43" t="s">
         <x:v>130</x:v>
-      </x:c>
-      <x:c r="C14" s="43" t="s">
-        <x:v>131</x:v>
       </x:c>
       <x:c r="D14" s="42">
         <x:v>8</x:v>
@@ -9254,7 +9251,7 @@
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="194" t="s">
-        <x:v>126</x:v>
+        <x:v>125</x:v>
       </x:c>
       <x:c r="B17" s="193"/>
       <x:c r="C17" s="193"/>
@@ -9298,7 +9295,7 @@
     </x:row>
     <x:row r="19" s="14" customFormat="1" ht="15.399999618530273" customHeight="1">
       <x:c r="A19" s="192" t="s">
-        <x:v>132</x:v>
+        <x:v>131</x:v>
       </x:c>
       <x:c r="B19" s="193"/>
       <x:c r="C19" s="193"/>
@@ -9312,10 +9309,10 @@
     </x:row>
     <x:row r="20">
       <x:c r="A20" s="40" t="s">
+        <x:v>120</x:v>
+      </x:c>
+      <x:c r="B20" s="40" t="s">
         <x:v>121</x:v>
-      </x:c>
-      <x:c r="B20" s="40" t="s">
-        <x:v>122</x:v>
       </x:c>
       <x:c r="C20" s="40" t="s">
         <x:v>14</x:v>
@@ -9330,7 +9327,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G20" s="40" t="s">
-        <x:v>123</x:v>
+        <x:v>122</x:v>
       </x:c>
       <x:c r="H20" s="40" t="s">
         <x:v>6</x:v>
@@ -9371,10 +9368,10 @@
         <x:v>43</x:v>
       </x:c>
       <x:c r="B23" s="41" t="s">
+        <x:v>132</x:v>
+      </x:c>
+      <x:c r="C23" s="43" t="s">
         <x:v>133</x:v>
-      </x:c>
-      <x:c r="C23" s="43" t="s">
-        <x:v>134</x:v>
       </x:c>
       <x:c r="D23" s="42">
         <x:v>7</x:v>
@@ -9401,10 +9398,10 @@
         <x:v>74</x:v>
       </x:c>
       <x:c r="B24" s="41" t="s">
+        <x:v>134</x:v>
+      </x:c>
+      <x:c r="C24" s="43" t="s">
         <x:v>135</x:v>
-      </x:c>
-      <x:c r="C24" s="43" t="s">
-        <x:v>136</x:v>
       </x:c>
       <x:c r="D24" s="42">
         <x:v>3</x:v>
@@ -9431,10 +9428,10 @@
         <x:v>45</x:v>
       </x:c>
       <x:c r="B25" s="41" t="s">
+        <x:v>136</x:v>
+      </x:c>
+      <x:c r="C25" s="43" t="s">
         <x:v>137</x:v>
-      </x:c>
-      <x:c r="C25" s="43" t="s">
-        <x:v>138</x:v>
       </x:c>
       <x:c r="D25" s="42">
         <x:v>4</x:v>
@@ -9461,10 +9458,10 @@
         <x:v>21</x:v>
       </x:c>
       <x:c r="B26" s="41" t="s">
+        <x:v>138</x:v>
+      </x:c>
+      <x:c r="C26" s="43" t="s">
         <x:v>139</x:v>
-      </x:c>
-      <x:c r="C26" s="43" t="s">
-        <x:v>140</x:v>
       </x:c>
       <x:c r="D26" s="42">
         <x:v>2</x:v>
@@ -9520,7 +9517,7 @@
     </x:row>
     <x:row r="28">
       <x:c r="A28" s="194" t="s">
-        <x:v>126</x:v>
+        <x:v>125</x:v>
       </x:c>
       <x:c r="B28" s="193"/>
       <x:c r="C28" s="193"/>
@@ -9564,7 +9561,7 @@
     </x:row>
     <x:row r="30" s="14" customFormat="1" ht="15.399999618530273" customHeight="1">
       <x:c r="A30" s="192" t="s">
-        <x:v>141</x:v>
+        <x:v>140</x:v>
       </x:c>
       <x:c r="B30" s="193"/>
       <x:c r="C30" s="193"/>
@@ -9578,10 +9575,10 @@
     </x:row>
     <x:row r="31">
       <x:c r="A31" s="40" t="s">
+        <x:v>120</x:v>
+      </x:c>
+      <x:c r="B31" s="40" t="s">
         <x:v>121</x:v>
-      </x:c>
-      <x:c r="B31" s="40" t="s">
-        <x:v>122</x:v>
       </x:c>
       <x:c r="C31" s="40" t="s">
         <x:v>14</x:v>
@@ -9596,7 +9593,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G31" s="40" t="s">
-        <x:v>123</x:v>
+        <x:v>122</x:v>
       </x:c>
       <x:c r="H31" s="40" t="s">
         <x:v>6</x:v>
@@ -9643,10 +9640,10 @@
         <x:v>33</x:v>
       </x:c>
       <x:c r="B33" s="42" t="s">
+        <x:v>141</x:v>
+      </x:c>
+      <x:c r="C33" s="43" t="s">
         <x:v>142</x:v>
-      </x:c>
-      <x:c r="C33" s="43" t="s">
-        <x:v>143</x:v>
       </x:c>
       <x:c r="D33" s="42">
         <x:v>5</x:v>
@@ -9685,10 +9682,10 @@
         <x:v>53</x:v>
       </x:c>
       <x:c r="B35" s="41" t="s">
+        <x:v>143</x:v>
+      </x:c>
+      <x:c r="C35" s="43" t="s">
         <x:v>144</x:v>
-      </x:c>
-      <x:c r="C35" s="43" t="s">
-        <x:v>145</x:v>
       </x:c>
       <x:c r="D35" s="42">
         <x:v>2</x:v>
@@ -9715,10 +9712,10 @@
         <x:v>41</x:v>
       </x:c>
       <x:c r="B36" s="41" t="s">
-        <x:v>124</x:v>
+        <x:v>123</x:v>
       </x:c>
       <x:c r="C36" s="43" t="s">
-        <x:v>146</x:v>
+        <x:v>145</x:v>
       </x:c>
       <x:c r="D36" s="42">
         <x:v>2</x:v>
@@ -9745,10 +9742,10 @@
         <x:v>41</x:v>
       </x:c>
       <x:c r="B37" s="42" t="s">
-        <x:v>142</x:v>
+        <x:v>141</x:v>
       </x:c>
       <x:c r="C37" s="43" t="s">
-        <x:v>147</x:v>
+        <x:v>146</x:v>
       </x:c>
       <x:c r="D37" s="42">
         <x:v>4</x:v>
@@ -9804,7 +9801,7 @@
     </x:row>
     <x:row r="39">
       <x:c r="A39" s="194" t="s">
-        <x:v>126</x:v>
+        <x:v>125</x:v>
       </x:c>
       <x:c r="B39" s="193"/>
       <x:c r="C39" s="193"/>
@@ -9848,7 +9845,7 @@
     </x:row>
     <x:row r="41" s="14" customFormat="1" ht="15.399999618530273" customHeight="1">
       <x:c r="A41" s="192" t="s">
-        <x:v>148</x:v>
+        <x:v>147</x:v>
       </x:c>
       <x:c r="B41" s="193"/>
       <x:c r="C41" s="193"/>
@@ -9862,10 +9859,10 @@
     </x:row>
     <x:row r="42">
       <x:c r="A42" s="40" t="s">
+        <x:v>120</x:v>
+      </x:c>
+      <x:c r="B42" s="40" t="s">
         <x:v>121</x:v>
-      </x:c>
-      <x:c r="B42" s="40" t="s">
-        <x:v>122</x:v>
       </x:c>
       <x:c r="C42" s="40" t="s">
         <x:v>14</x:v>
@@ -9880,7 +9877,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G42" s="40" t="s">
-        <x:v>123</x:v>
+        <x:v>122</x:v>
       </x:c>
       <x:c r="H42" s="40" t="s">
         <x:v>6</x:v>
@@ -9897,10 +9894,10 @@
         <x:v>66</x:v>
       </x:c>
       <x:c r="B43" s="38" t="s">
-        <x:v>139</x:v>
+        <x:v>138</x:v>
       </x:c>
       <x:c r="C43" s="38" t="s">
-        <x:v>149</x:v>
+        <x:v>148</x:v>
       </x:c>
       <x:c r="D43" s="49">
         <x:v>4</x:v>
@@ -9927,10 +9924,10 @@
         <x:v>69</x:v>
       </x:c>
       <x:c r="B44" s="41" t="s">
+        <x:v>149</x:v>
+      </x:c>
+      <x:c r="C44" s="43" t="s">
         <x:v>150</x:v>
-      </x:c>
-      <x:c r="C44" s="43" t="s">
-        <x:v>151</x:v>
       </x:c>
       <x:c r="D44" s="42">
         <x:v>4</x:v>
@@ -9987,10 +9984,10 @@
         <x:v>58</x:v>
       </x:c>
       <x:c r="B46" s="41" t="s">
+        <x:v>151</x:v>
+      </x:c>
+      <x:c r="C46" s="43" t="s">
         <x:v>152</x:v>
-      </x:c>
-      <x:c r="C46" s="43" t="s">
-        <x:v>153</x:v>
       </x:c>
       <x:c r="D46" s="42">
         <x:v>5</x:v>
@@ -10046,7 +10043,7 @@
     </x:row>
     <x:row r="48">
       <x:c r="A48" s="194" t="s">
-        <x:v>126</x:v>
+        <x:v>125</x:v>
       </x:c>
       <x:c r="B48" s="193"/>
       <x:c r="C48" s="193"/>
@@ -10090,7 +10087,7 @@
     </x:row>
     <x:row r="50" s="14" customFormat="1" ht="15.399999618530273" customHeight="1">
       <x:c r="A50" s="192" t="s">
-        <x:v>154</x:v>
+        <x:v>153</x:v>
       </x:c>
       <x:c r="B50" s="193"/>
       <x:c r="C50" s="193"/>
@@ -10104,10 +10101,10 @@
     </x:row>
     <x:row r="51">
       <x:c r="A51" s="40" t="s">
+        <x:v>120</x:v>
+      </x:c>
+      <x:c r="B51" s="40" t="s">
         <x:v>121</x:v>
-      </x:c>
-      <x:c r="B51" s="40" t="s">
-        <x:v>122</x:v>
       </x:c>
       <x:c r="C51" s="40" t="s">
         <x:v>14</x:v>
@@ -10122,7 +10119,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G51" s="40" t="s">
-        <x:v>123</x:v>
+        <x:v>122</x:v>
       </x:c>
       <x:c r="H51" s="40" t="s">
         <x:v>6</x:v>
@@ -10139,10 +10136,10 @@
         <x:v>70</x:v>
       </x:c>
       <x:c r="B52" s="38" t="s">
-        <x:v>152</x:v>
+        <x:v>151</x:v>
       </x:c>
       <x:c r="C52" s="38" t="s">
-        <x:v>155</x:v>
+        <x:v>154</x:v>
       </x:c>
       <x:c r="D52" s="49">
         <x:v>4</x:v>
@@ -10169,10 +10166,10 @@
         <x:v>37</x:v>
       </x:c>
       <x:c r="B53" s="42" t="s">
+        <x:v>155</x:v>
+      </x:c>
+      <x:c r="C53" s="43" t="s">
         <x:v>156</x:v>
-      </x:c>
-      <x:c r="C53" s="43" t="s">
-        <x:v>157</x:v>
       </x:c>
       <x:c r="D53" s="42">
         <x:v>6</x:v>
@@ -10199,10 +10196,10 @@
         <x:v>71</x:v>
       </x:c>
       <x:c r="B54" s="42" t="s">
+        <x:v>157</x:v>
+      </x:c>
+      <x:c r="C54" s="43" t="s">
         <x:v>158</x:v>
-      </x:c>
-      <x:c r="C54" s="43" t="s">
-        <x:v>159</x:v>
       </x:c>
       <x:c r="D54" s="42">
         <x:v>1</x:v>
@@ -10229,10 +10226,10 @@
         <x:v>72</x:v>
       </x:c>
       <x:c r="B55" s="41" t="s">
+        <x:v>159</x:v>
+      </x:c>
+      <x:c r="C55" s="43" t="s">
         <x:v>160</x:v>
-      </x:c>
-      <x:c r="C55" s="43" t="s">
-        <x:v>161</x:v>
       </x:c>
       <x:c r="D55" s="42">
         <x:v>3</x:v>
@@ -10259,10 +10256,10 @@
         <x:v>49</x:v>
       </x:c>
       <x:c r="B56" s="42" t="s">
+        <x:v>161</x:v>
+      </x:c>
+      <x:c r="C56" s="43" t="s">
         <x:v>162</x:v>
-      </x:c>
-      <x:c r="C56" s="43" t="s">
-        <x:v>163</x:v>
       </x:c>
       <x:c r="D56" s="42">
         <x:v>2</x:v>
@@ -10289,10 +10286,10 @@
         <x:v>65</x:v>
       </x:c>
       <x:c r="B57" s="41" t="s">
+        <x:v>163</x:v>
+      </x:c>
+      <x:c r="C57" s="43" t="s">
         <x:v>164</x:v>
-      </x:c>
-      <x:c r="C57" s="43" t="s">
-        <x:v>165</x:v>
       </x:c>
       <x:c r="D57" s="42">
         <x:v>4</x:v>
@@ -10319,10 +10316,10 @@
         <x:v>67</x:v>
       </x:c>
       <x:c r="B58" s="41" t="s">
+        <x:v>165</x:v>
+      </x:c>
+      <x:c r="C58" s="43" t="s">
         <x:v>166</x:v>
-      </x:c>
-      <x:c r="C58" s="43" t="s">
-        <x:v>167</x:v>
       </x:c>
       <x:c r="D58" s="42">
         <x:v>7</x:v>
@@ -10349,10 +10346,10 @@
         <x:v>68</x:v>
       </x:c>
       <x:c r="B59" s="42" t="s">
-        <x:v>142</x:v>
+        <x:v>141</x:v>
       </x:c>
       <x:c r="C59" s="43" t="s">
-        <x:v>168</x:v>
+        <x:v>167</x:v>
       </x:c>
       <x:c r="D59" s="42">
         <x:v>4</x:v>
@@ -10379,10 +10376,10 @@
         <x:v>65</x:v>
       </x:c>
       <x:c r="B60" s="42" t="s">
+        <x:v>168</x:v>
+      </x:c>
+      <x:c r="C60" s="43" t="s">
         <x:v>169</x:v>
-      </x:c>
-      <x:c r="C60" s="43" t="s">
-        <x:v>170</x:v>
       </x:c>
       <x:c r="D60" s="42">
         <x:v>6</x:v>
@@ -10409,10 +10406,10 @@
         <x:v>66</x:v>
       </x:c>
       <x:c r="B61" s="41" t="s">
+        <x:v>170</x:v>
+      </x:c>
+      <x:c r="C61" s="43" t="s">
         <x:v>171</x:v>
-      </x:c>
-      <x:c r="C61" s="43" t="s">
-        <x:v>172</x:v>
       </x:c>
       <x:c r="D61" s="42">
         <x:v>2</x:v>
@@ -10439,10 +10436,10 @@
         <x:v>35</x:v>
       </x:c>
       <x:c r="B62" s="42" t="s">
+        <x:v>172</x:v>
+      </x:c>
+      <x:c r="C62" s="43" t="s">
         <x:v>173</x:v>
-      </x:c>
-      <x:c r="C62" s="43" t="s">
-        <x:v>174</x:v>
       </x:c>
       <x:c r="D62" s="42">
         <x:v>3</x:v>
@@ -10528,7 +10525,7 @@
     </x:row>
     <x:row r="65">
       <x:c r="A65" s="194" t="s">
-        <x:v>126</x:v>
+        <x:v>125</x:v>
       </x:c>
       <x:c r="B65" s="193"/>
       <x:c r="C65" s="193"/>
@@ -10572,7 +10569,7 @@
     </x:row>
     <x:row r="67" s="14" customFormat="1" ht="15.399999618530273" customHeight="1">
       <x:c r="A67" s="192" t="s">
-        <x:v>175</x:v>
+        <x:v>174</x:v>
       </x:c>
       <x:c r="B67" s="193"/>
       <x:c r="C67" s="193"/>
@@ -10586,10 +10583,10 @@
     </x:row>
     <x:row r="68">
       <x:c r="A68" s="40" t="s">
+        <x:v>120</x:v>
+      </x:c>
+      <x:c r="B68" s="40" t="s">
         <x:v>121</x:v>
-      </x:c>
-      <x:c r="B68" s="40" t="s">
-        <x:v>122</x:v>
       </x:c>
       <x:c r="C68" s="40" t="s">
         <x:v>14</x:v>
@@ -10604,7 +10601,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G68" s="40" t="s">
-        <x:v>123</x:v>
+        <x:v>122</x:v>
       </x:c>
       <x:c r="H68" s="40" t="s">
         <x:v>6</x:v>
@@ -10633,10 +10630,10 @@
         <x:v>66</x:v>
       </x:c>
       <x:c r="B70" s="42" t="s">
-        <x:v>142</x:v>
+        <x:v>141</x:v>
       </x:c>
       <x:c r="C70" s="43" t="s">
-        <x:v>176</x:v>
+        <x:v>175</x:v>
       </x:c>
       <x:c r="D70" s="42">
         <x:v>4</x:v>
@@ -10660,13 +10657,13 @@
     </x:row>
     <x:row r="71" ht="17.25">
       <x:c r="A71" s="41" t="s">
+        <x:v>176</x:v>
+      </x:c>
+      <x:c r="B71" s="41" t="s">
         <x:v>177</x:v>
       </x:c>
-      <x:c r="B71" s="41" t="s">
+      <x:c r="C71" s="43" t="s">
         <x:v>178</x:v>
-      </x:c>
-      <x:c r="C71" s="43" t="s">
-        <x:v>179</x:v>
       </x:c>
       <x:c r="D71" s="42">
         <x:v>1</x:v>
@@ -10693,10 +10690,10 @@
         <x:v>23</x:v>
       </x:c>
       <x:c r="B72" s="51" t="s">
+        <x:v>179</x:v>
+      </x:c>
+      <x:c r="C72" s="51" t="s">
         <x:v>180</x:v>
-      </x:c>
-      <x:c r="C72" s="51" t="s">
-        <x:v>181</x:v>
       </x:c>
       <x:c r="D72" s="52">
         <x:v>1</x:v>
@@ -10723,10 +10720,10 @@
         <x:v>87</x:v>
       </x:c>
       <x:c r="B73" s="48" t="s">
+        <x:v>181</x:v>
+      </x:c>
+      <x:c r="C73" s="48" t="s">
         <x:v>182</x:v>
-      </x:c>
-      <x:c r="C73" s="48" t="s">
-        <x:v>183</x:v>
       </x:c>
       <x:c r="D73" s="53">
         <x:v>3</x:v>
@@ -10782,7 +10779,7 @@
     </x:row>
     <x:row r="75" s="14" customFormat="1" ht="15.399999618530273" customHeight="1">
       <x:c r="A75" s="56" t="s">
-        <x:v>126</x:v>
+        <x:v>125</x:v>
       </x:c>
       <x:c r="B75" s="48"/>
       <x:c r="C75" s="48"/>
@@ -10814,7 +10811,7 @@
     </x:row>
     <x:row r="76" s="14" customFormat="1" ht="19.149999618530273" customHeight="1">
       <x:c r="A76" s="198" t="s">
-        <x:v>184</x:v>
+        <x:v>183</x:v>
       </x:c>
       <x:c r="B76" s="193"/>
       <x:c r="C76" s="193"/>
@@ -10828,10 +10825,10 @@
     </x:row>
     <x:row r="77" s="14" customFormat="1" ht="19.149999618530273" customHeight="1">
       <x:c r="A77" s="57" t="s">
+        <x:v>120</x:v>
+      </x:c>
+      <x:c r="B77" s="58" t="s">
         <x:v>121</x:v>
-      </x:c>
-      <x:c r="B77" s="58" t="s">
-        <x:v>122</x:v>
       </x:c>
       <x:c r="C77" s="58" t="s">
         <x:v>14</x:v>
@@ -10846,7 +10843,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G77" s="59" t="s">
-        <x:v>123</x:v>
+        <x:v>122</x:v>
       </x:c>
       <x:c r="H77" s="59" t="s">
         <x:v>6</x:v>
@@ -10863,10 +10860,10 @@
         <x:v>29</x:v>
       </x:c>
       <x:c r="B78" s="38" t="s">
-        <x:v>128</x:v>
+        <x:v>127</x:v>
       </x:c>
       <x:c r="C78" s="38" t="s">
-        <x:v>185</x:v>
+        <x:v>184</x:v>
       </x:c>
       <x:c r="D78" s="50">
         <x:v>4</x:v>
@@ -10893,10 +10890,10 @@
         <x:v>78</x:v>
       </x:c>
       <x:c r="B79" s="38" t="s">
-        <x:v>124</x:v>
+        <x:v>123</x:v>
       </x:c>
       <x:c r="C79" s="38" t="s">
-        <x:v>186</x:v>
+        <x:v>185</x:v>
       </x:c>
       <x:c r="D79" s="50">
         <x:v>2</x:v>
@@ -10923,10 +10920,10 @@
         <x:v>23</x:v>
       </x:c>
       <x:c r="B80" s="41" t="s">
+        <x:v>186</x:v>
+      </x:c>
+      <x:c r="C80" s="43" t="s">
         <x:v>187</x:v>
-      </x:c>
-      <x:c r="C80" s="43" t="s">
-        <x:v>188</x:v>
       </x:c>
       <x:c r="D80" s="42">
         <x:v>3</x:v>
@@ -10953,10 +10950,10 @@
         <x:v>49</x:v>
       </x:c>
       <x:c r="B81" s="41" t="s">
+        <x:v>188</x:v>
+      </x:c>
+      <x:c r="C81" s="43" t="s">
         <x:v>189</x:v>
-      </x:c>
-      <x:c r="C81" s="43" t="s">
-        <x:v>190</x:v>
       </x:c>
       <x:c r="D81" s="42">
         <x:v>5</x:v>
@@ -10983,10 +10980,10 @@
         <x:v>53</x:v>
       </x:c>
       <x:c r="B82" s="41" t="s">
+        <x:v>190</x:v>
+      </x:c>
+      <x:c r="C82" s="43" t="s">
         <x:v>191</x:v>
-      </x:c>
-      <x:c r="C82" s="43" t="s">
-        <x:v>192</x:v>
       </x:c>
       <x:c r="D82" s="42">
         <x:v>3</x:v>
@@ -11025,10 +11022,10 @@
         <x:v>37</x:v>
       </x:c>
       <x:c r="B84" s="41" t="s">
+        <x:v>192</x:v>
+      </x:c>
+      <x:c r="C84" s="43" t="s">
         <x:v>193</x:v>
-      </x:c>
-      <x:c r="C84" s="43" t="s">
-        <x:v>194</x:v>
       </x:c>
       <x:c r="D84" s="42">
         <x:v>3</x:v>
@@ -11096,7 +11093,7 @@
     </x:row>
     <x:row r="87">
       <x:c r="A87" s="48" t="s">
-        <x:v>126</x:v>
+        <x:v>125</x:v>
       </x:c>
       <x:c r="B87" s="48"/>
       <x:c r="C87" s="48"/>
@@ -11140,7 +11137,7 @@
     </x:row>
     <x:row r="89" s="14" customFormat="1" ht="19.149999618530273" customHeight="1">
       <x:c r="A89" s="198" t="s">
-        <x:v>195</x:v>
+        <x:v>194</x:v>
       </x:c>
       <x:c r="B89" s="193"/>
       <x:c r="C89" s="193"/>
@@ -11154,10 +11151,10 @@
     </x:row>
     <x:row r="90" s="14" customFormat="1" ht="19.149999618530273" customHeight="1">
       <x:c r="A90" s="59" t="s">
+        <x:v>120</x:v>
+      </x:c>
+      <x:c r="B90" s="58" t="s">
         <x:v>121</x:v>
-      </x:c>
-      <x:c r="B90" s="58" t="s">
-        <x:v>122</x:v>
       </x:c>
       <x:c r="C90" s="58" t="s">
         <x:v>14</x:v>
@@ -11172,7 +11169,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G90" s="59" t="s">
-        <x:v>123</x:v>
+        <x:v>122</x:v>
       </x:c>
       <x:c r="H90" s="59" t="s">
         <x:v>6</x:v>
@@ -11189,10 +11186,10 @@
         <x:v>33</x:v>
       </x:c>
       <x:c r="B91" s="38" t="s">
+        <x:v>195</x:v>
+      </x:c>
+      <x:c r="C91" s="38" t="s">
         <x:v>196</x:v>
-      </x:c>
-      <x:c r="C91" s="38" t="s">
-        <x:v>197</x:v>
       </x:c>
       <x:c r="D91" s="65">
         <x:v>6</x:v>
@@ -11213,7 +11210,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="J91" s="44" t="s">
-        <x:v>198</x:v>
+        <x:v>197</x:v>
       </x:c>
     </x:row>
     <x:row r="92">
@@ -11221,10 +11218,10 @@
         <x:v>82</x:v>
       </x:c>
       <x:c r="B92" s="38" t="s">
+        <x:v>198</x:v>
+      </x:c>
+      <x:c r="C92" s="38" t="s">
         <x:v>199</x:v>
-      </x:c>
-      <x:c r="C92" s="38" t="s">
-        <x:v>200</x:v>
       </x:c>
       <x:c r="D92" s="50">
         <x:v>4</x:v>
@@ -11251,10 +11248,10 @@
         <x:v>68</x:v>
       </x:c>
       <x:c r="B93" s="41" t="s">
+        <x:v>200</x:v>
+      </x:c>
+      <x:c r="C93" s="43" t="s">
         <x:v>201</x:v>
-      </x:c>
-      <x:c r="C93" s="43" t="s">
-        <x:v>202</x:v>
       </x:c>
       <x:c r="D93" s="42">
         <x:v>4</x:v>
@@ -11281,10 +11278,10 @@
         <x:v>68</x:v>
       </x:c>
       <x:c r="B94" s="41" t="s">
+        <x:v>202</x:v>
+      </x:c>
+      <x:c r="C94" s="43" t="s">
         <x:v>203</x:v>
-      </x:c>
-      <x:c r="C94" s="43" t="s">
-        <x:v>204</x:v>
       </x:c>
       <x:c r="D94" s="42">
         <x:v>5</x:v>
@@ -11305,7 +11302,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="J94" s="68" t="s">
-        <x:v>205</x:v>
+        <x:v>204</x:v>
       </x:c>
     </x:row>
     <x:row r="95" ht="17.25">
@@ -11313,7 +11310,7 @@
         <x:v>33</x:v>
       </x:c>
       <x:c r="B95" s="41" t="s">
-        <x:v>196</x:v>
+        <x:v>195</x:v>
       </x:c>
       <x:c r="C95" s="43" t="s">
         <x:v>54</x:v>
@@ -11337,7 +11334,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="J95" s="44" t="s">
-        <x:v>206</x:v>
+        <x:v>205</x:v>
       </x:c>
     </x:row>
     <x:row r="96">
@@ -11345,10 +11342,10 @@
         <x:v>79</x:v>
       </x:c>
       <x:c r="B96" s="42" t="s">
-        <x:v>144</x:v>
+        <x:v>143</x:v>
       </x:c>
       <x:c r="C96" s="43" t="s">
-        <x:v>207</x:v>
+        <x:v>206</x:v>
       </x:c>
       <x:c r="D96" s="42">
         <x:v>4</x:v>
@@ -11375,10 +11372,10 @@
         <x:v>81</x:v>
       </x:c>
       <x:c r="B97" s="41" t="s">
+        <x:v>207</x:v>
+      </x:c>
+      <x:c r="C97" s="43" t="s">
         <x:v>208</x:v>
-      </x:c>
-      <x:c r="C97" s="43" t="s">
-        <x:v>209</x:v>
       </x:c>
       <x:c r="D97" s="42">
         <x:v>5</x:v>
@@ -11399,7 +11396,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="J97" s="44" t="s">
-        <x:v>206</x:v>
+        <x:v>205</x:v>
       </x:c>
     </x:row>
     <x:row r="98" ht="17.25">
@@ -11407,10 +11404,10 @@
         <x:v>80</x:v>
       </x:c>
       <x:c r="B98" s="41" t="s">
+        <x:v>209</x:v>
+      </x:c>
+      <x:c r="C98" s="43" t="s">
         <x:v>210</x:v>
-      </x:c>
-      <x:c r="C98" s="43" t="s">
-        <x:v>211</x:v>
       </x:c>
       <x:c r="D98" s="42">
         <x:v>1</x:v>
@@ -11437,10 +11434,10 @@
         <x:v>82</x:v>
       </x:c>
       <x:c r="B99" s="48" t="s">
+        <x:v>211</x:v>
+      </x:c>
+      <x:c r="C99" s="48" t="s">
         <x:v>212</x:v>
-      </x:c>
-      <x:c r="C99" s="48" t="s">
-        <x:v>213</x:v>
       </x:c>
       <x:c r="D99" s="53">
         <x:v>3</x:v>
@@ -11467,10 +11464,10 @@
         <x:v>80</x:v>
       </x:c>
       <x:c r="B100" s="44" t="s">
+        <x:v>213</x:v>
+      </x:c>
+      <x:c r="C100" s="44" t="s">
         <x:v>214</x:v>
-      </x:c>
-      <x:c r="C100" s="44" t="s">
-        <x:v>215</x:v>
       </x:c>
       <x:c r="D100" s="53">
         <x:v>1</x:v>
@@ -11523,12 +11520,12 @@
         <x:v>12</x:v>
       </x:c>
       <x:c r="J101" s="61" t="s">
-        <x:v>216</x:v>
+        <x:v>215</x:v>
       </x:c>
     </x:row>
     <x:row r="102" s="14" customFormat="1" ht="15.399999618530273" customHeight="1">
       <x:c r="A102" s="48" t="s">
-        <x:v>126</x:v>
+        <x:v>125</x:v>
       </x:c>
       <x:c r="B102" s="48"/>
       <x:c r="C102" s="48"/>
@@ -11572,7 +11569,7 @@
     </x:row>
     <x:row r="104" s="14" customFormat="1" ht="19.149999618530273" customHeight="1">
       <x:c r="A104" s="72" t="s">
-        <x:v>217</x:v>
+        <x:v>216</x:v>
       </x:c>
       <x:c r="B104" s="44"/>
       <x:c r="C104" s="44"/>
@@ -11586,10 +11583,10 @@
     </x:row>
     <x:row r="105">
       <x:c r="A105" s="59" t="s">
+        <x:v>120</x:v>
+      </x:c>
+      <x:c r="B105" s="57" t="s">
         <x:v>121</x:v>
-      </x:c>
-      <x:c r="B105" s="57" t="s">
-        <x:v>122</x:v>
       </x:c>
       <x:c r="C105" s="57" t="s">
         <x:v>14</x:v>
@@ -11604,7 +11601,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G105" s="59" t="s">
-        <x:v>123</x:v>
+        <x:v>122</x:v>
       </x:c>
       <x:c r="H105" s="59" t="s">
         <x:v>6</x:v>
@@ -11621,10 +11618,10 @@
         <x:v>85</x:v>
       </x:c>
       <x:c r="B106" s="41" t="s">
+        <x:v>217</x:v>
+      </x:c>
+      <x:c r="C106" s="43" t="s">
         <x:v>218</x:v>
-      </x:c>
-      <x:c r="C106" s="43" t="s">
-        <x:v>219</x:v>
       </x:c>
       <x:c r="D106" s="42">
         <x:v>4</x:v>
@@ -11648,13 +11645,13 @@
     </x:row>
     <x:row r="107">
       <x:c r="A107" s="42" t="s">
+        <x:v>219</x:v>
+      </x:c>
+      <x:c r="B107" s="41" t="s">
         <x:v>220</x:v>
       </x:c>
-      <x:c r="B107" s="41" t="s">
+      <x:c r="C107" s="43" t="s">
         <x:v>221</x:v>
-      </x:c>
-      <x:c r="C107" s="43" t="s">
-        <x:v>222</x:v>
       </x:c>
       <x:c r="D107" s="42">
         <x:v>4</x:v>
@@ -11681,10 +11678,10 @@
         <x:v>35</x:v>
       </x:c>
       <x:c r="B108" s="41" t="s">
+        <x:v>222</x:v>
+      </x:c>
+      <x:c r="C108" s="43" t="s">
         <x:v>223</x:v>
-      </x:c>
-      <x:c r="C108" s="43" t="s">
-        <x:v>224</x:v>
       </x:c>
       <x:c r="D108" s="42">
         <x:v>3</x:v>
@@ -11708,13 +11705,13 @@
     </x:row>
     <x:row r="109" ht="21">
       <x:c r="A109" s="60" t="s">
+        <x:v>224</x:v>
+      </x:c>
+      <x:c r="B109" s="44" t="s">
+        <x:v>198</x:v>
+      </x:c>
+      <x:c r="C109" s="44" t="s">
         <x:v>225</x:v>
-      </x:c>
-      <x:c r="B109" s="44" t="s">
-        <x:v>199</x:v>
-      </x:c>
-      <x:c r="C109" s="44" t="s">
-        <x:v>226</x:v>
       </x:c>
       <x:c r="D109" s="53">
         <x:v>4</x:v>
@@ -11735,7 +11732,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="J109" s="69" t="s">
-        <x:v>206</x:v>
+        <x:v>205</x:v>
       </x:c>
     </x:row>
     <x:row r="110" ht="18.75">
@@ -11743,7 +11740,7 @@
         <x:v>56</x:v>
       </x:c>
       <x:c r="B110" s="44" t="s">
-        <x:v>227</x:v>
+        <x:v>226</x:v>
       </x:c>
       <x:c r="C110" s="44" t="s">
         <x:v>55</x:v>
@@ -11773,7 +11770,7 @@
         <x:v>58</x:v>
       </x:c>
       <x:c r="B111" s="129" t="s">
-        <x:v>228</x:v>
+        <x:v>227</x:v>
       </x:c>
       <x:c r="C111" s="129" t="s">
         <x:v>57</x:v>
@@ -11803,10 +11800,10 @@
         <x:v>73</x:v>
       </x:c>
       <x:c r="B112" s="173" t="s">
-        <x:v>196</x:v>
+        <x:v>195</x:v>
       </x:c>
       <x:c r="C112" s="173" t="s">
-        <x:v>229</x:v>
+        <x:v>228</x:v>
       </x:c>
       <x:c r="D112" s="174">
         <x:v>8</x:v>
@@ -11833,7 +11830,7 @@
         <x:v>33</x:v>
       </x:c>
       <x:c r="B113" s="175" t="s">
-        <x:v>150</x:v>
+        <x:v>149</x:v>
       </x:c>
       <x:c r="C113" s="175" t="s">
         <x:v>59</x:v>
@@ -11863,10 +11860,10 @@
         <x:v>43</x:v>
       </x:c>
       <x:c r="B114" s="176" t="s">
+        <x:v>229</x:v>
+      </x:c>
+      <x:c r="C114" s="176" t="s">
         <x:v>230</x:v>
-      </x:c>
-      <x:c r="C114" s="176" t="s">
-        <x:v>231</x:v>
       </x:c>
       <x:c r="D114" s="178">
         <x:v>2</x:v>
@@ -13173,6 +13170,6 @@
     <x:mergeCell ref="A50:T50"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra4bed8e122bc4f5c"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R24b884fc15174b5f"/>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Update TERA PROJECT under southern branch
</commit_message>
<xml_diff>
--- a/채용비율.xlsx
+++ b/채용비율.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1.26년 전체 소속별 점유율" sheetId="1" r:id="Rf9a42abcac194542"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2.각8개지부 현장점유율" sheetId="2" r:id="R575daa7d0bb2459a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3.타워사별 점유현황" sheetId="3" r:id="R51d5626cf6584477"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4.반도체현장" sheetId="4" r:id="R375fd11df0e240ae"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5.1~9월채용추이" sheetId="5" r:id="Ra1f275c8a34d4eab"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="6.월별 소속별 채용비율" sheetId="6" r:id="R118a5c739999476d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1.26년 전체 소속별 점유율" sheetId="1" r:id="R3bfcfa18851b4020"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2.각8개지부 현장점유율" sheetId="2" r:id="Ra506fe6d0c294a13"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3.타워사별 점유현황" sheetId="3" r:id="R31fec0e134334b05"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4.반도체현장" sheetId="4" r:id="Rdd9cc5e27810442a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5.1~9월채용추이" sheetId="5" r:id="R9fbc64cd003e4d74"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="6.월별 소속별 채용비율" sheetId="6" r:id="R4e5ecdfe5b234c19"/>
   </x:sheets>
   <x:definedNames>
     <x:definedName name="가평군">#REF!</x:definedName>
@@ -1524,7 +1524,7 @@
       <x:alignment vertical="center"/>
     </x:xf>
   </x:cellStyleXfs>
-  <x:cellXfs count="568">
+  <x:cellXfs count="570">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1">
       <x:alignment vertical="center"/>
     </x:xf>
@@ -3188,6 +3188,12 @@
     </x:xf>
     <x:xf numFmtId="200" fontId="6" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="45" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="176" fontId="45" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="4">
@@ -3414,7 +3420,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R0991f3956ad24826"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rf0c9f4501ca14137"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -3663,27 +3669,26 @@
       <x:c r="A3" s="8" t="s">
         <x:v>10</x:v>
       </x:c>
-      <x:c r="B3" s="567">
-        <x:v>72</x:v>
+      <x:c r="B3" s="567" t="n">
+        <x:v>73</x:v>
       </x:c>
       <x:c r="C3" s="567" t="n">
-        <x:v>106</x:v>
+        <x:v>107</x:v>
       </x:c>
       <x:c r="D3" s="567" t="n">
         <x:v>9</x:v>
       </x:c>
-      <x:c r="E3" s="567">
+      <x:c r="E3" s="567" t="n">
         <x:v>10</x:v>
       </x:c>
-      <x:c r="F3" s="567">
+      <x:c r="F3" s="567" t="n">
         <x:v>42</x:v>
       </x:c>
       <x:c r="G3" s="567" t="n">
-        <x:v>15</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="H3" s="567" t="n">
-        <x:f>SUM(B3:G3)</x:f>
-        <x:v>254</x:v>
+        <x:v>258</x:v>
       </x:c>
       <x:c r="I3" s="9" t="s">
         <x:v>11</x:v>
@@ -3695,27 +3700,27 @@
       </x:c>
       <x:c r="B4" s="32" t="n">
         <x:f>IF($H$3=0,0,B3/$H$3)</x:f>
-        <x:v>0.28346456692913385</x:v>
+        <x:v>0.28294573643410853</x:v>
       </x:c>
       <x:c r="C4" s="32" t="n">
         <x:f>IF($H$3=0,0,C3/$H$3)</x:f>
-        <x:v>0.41732283464566927</x:v>
+        <x:v>0.41472868217054265</x:v>
       </x:c>
       <x:c r="D4" s="32" t="n">
         <x:f>IF($H$3=0,0,D3/$H$3)</x:f>
-        <x:v>0.03543307086614173</x:v>
+        <x:v>0.03488372093023256</x:v>
       </x:c>
       <x:c r="E4" s="32" t="n">
         <x:f>IF($H$3=0,0,E3/$H$3)</x:f>
-        <x:v>0.03937007874015748</x:v>
+        <x:v>0.03875968992248062</x:v>
       </x:c>
       <x:c r="F4" s="32" t="n">
         <x:f>IF($H$3=0,0,F3/$H$3)</x:f>
-        <x:v>0.16535433070866143</x:v>
+        <x:v>0.16279069767441862</x:v>
       </x:c>
       <x:c r="G4" s="32" t="n">
         <x:f>IF($H$3=0,0,G3/$H$3)</x:f>
-        <x:v>0.05905511811023622</x:v>
+        <x:v>0.06589147286821706</x:v>
       </x:c>
     </x:row>
     <x:row r="9" s="14" customFormat="1" ht="21.200000762939453" customHeight="1"/>
@@ -4746,109 +4751,111 @@
     </x:row>
     <x:row r="27">
       <x:c r="A27" s="38" t="str">
-        <x:v>남부지부 소계</x:v>
-      </x:c>
-      <x:c r="B27" s="38"/>
-      <x:c r="C27" s="38"/>
-      <x:c r="D27" s="38"/>
+        <x:v>남부</x:v>
+      </x:c>
+      <x:c r="B27" s="38" t="str">
+        <x:v>TERA PROJECT</x:v>
+      </x:c>
+      <x:c r="C27" s="38" t="str">
+        <x:v>(주)규람타워렌탈</x:v>
+      </x:c>
+      <x:c r="D27" s="38" t="str">
+        <x:v>원청사: 두산에너빌리티(주) / 2026-10-21 신규</x:v>
+      </x:c>
       <x:c r="E27" s="540" t="n">
-        <x:f>SUM(E8:E26)</x:f>
-        <x:v>23</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="F27" s="540" t="n">
-        <x:f>SUM(F8:F26)</x:f>
-        <x:v>41</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="G27" s="540" t="n">
-        <x:f>SUM(G8:G26)</x:f>
-        <x:v>2</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="H27" s="540" t="n">
-        <x:f>SUM(H8:H26)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I27" s="540" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J27" s="540" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="K27" s="540" t="n">
         <x:v>4</x:v>
-      </x:c>
-      <x:c r="I27" s="540" t="n">
-        <x:f>SUM(I8:I26)</x:f>
-        <x:v>14</x:v>
-      </x:c>
-      <x:c r="J27" s="540" t="n">
-        <x:f>SUM(J8:J26)</x:f>
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="K27" s="540" t="n">
-        <x:f>SUM(K8:K26)</x:f>
-        <x:v>87</x:v>
       </x:c>
       <x:c r="L27" s="38"/>
     </x:row>
     <x:row r="28" s="14" customFormat="1">
       <x:c r="A28" s="86" t="str">
-        <x:v>소계퍼센테이지</x:v>
+        <x:v>남부지부 소계</x:v>
       </x:c>
       <x:c r="B28" s="86"/>
       <x:c r="C28" s="86"/>
       <x:c r="D28" s="86"/>
-      <x:c r="E28" s="150" t="n">
-        <x:f>IF($K$27=0,0,E27/$K$27)</x:f>
-        <x:v>0.26436781609195403</x:v>
-      </x:c>
-      <x:c r="F28" s="150" t="n">
-        <x:f>IF($K$27=0,0,F27/$K$27)</x:f>
-        <x:v>0.47126436781609193</x:v>
-      </x:c>
-      <x:c r="G28" s="150" t="n">
-        <x:f>IF($K$27=0,0,G27/$K$27)</x:f>
-        <x:v>0.022988505747126436</x:v>
-      </x:c>
-      <x:c r="H28" s="150" t="n">
-        <x:f>IF($K$27=0,0,H27/$K$27)</x:f>
-        <x:v>0.04597701149425287</x:v>
-      </x:c>
-      <x:c r="I28" s="150" t="n">
-        <x:f>IF($K$27=0,0,I27/$K$27)</x:f>
-        <x:v>0.16091954022988506</x:v>
-      </x:c>
-      <x:c r="J28" s="150" t="n">
-        <x:f>IF($K$27=0,0,J27/$K$27)</x:f>
-        <x:v>0.034482758620689655</x:v>
-      </x:c>
-      <x:c r="K28" s="150" t="n">
-        <x:f>IF($K$27=0,0,K27/$K$27)</x:f>
-        <x:v>1</x:v>
+      <x:c r="E28" s="540" t="n">
+        <x:f>SUM(E8:E27)</x:f>
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="F28" s="540" t="n">
+        <x:f>SUM(F8:F27)</x:f>
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="G28" s="540" t="n">
+        <x:f>SUM(G8:G27)</x:f>
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="H28" s="540" t="n">
+        <x:f>SUM(H8:H27)</x:f>
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="I28" s="540" t="n">
+        <x:f>SUM(I8:I27)</x:f>
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="J28" s="540" t="n">
+        <x:f>SUM(J8:J27)</x:f>
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="K28" s="540" t="n">
+        <x:f>SUM(K8:K27)</x:f>
+        <x:v>91</x:v>
       </x:c>
       <x:c r="L28" s="86"/>
     </x:row>
     <x:row r="29" s="14" customFormat="1" ht="17.25">
       <x:c r="A29" s="83" t="str">
-        <x:v>남서</x:v>
-      </x:c>
-      <x:c r="B29" s="84" t="str">
-        <x:v>남양우미린</x:v>
-      </x:c>
-      <x:c r="C29" s="84" t="str">
-        <x:v>뉴월드타워 주식회사</x:v>
-      </x:c>
+        <x:v>소계퍼센테이지</x:v>
+      </x:c>
+      <x:c r="B29" s="84"/>
+      <x:c r="C29" s="84"/>
       <x:c r="D29" s="84"/>
-      <x:c r="E29" s="545" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="F29" s="545" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="G29" s="545" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="H29" s="545" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="I29" s="545" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="J29" s="545" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="K29" s="545" t="n">
-        <x:v>3</x:v>
+      <x:c r="E29" s="565" t="n">
+        <x:f>IF($K$28=0,0,E28/$K$28)</x:f>
+        <x:v>0.26373626373626374</x:v>
+      </x:c>
+      <x:c r="F29" s="565" t="n">
+        <x:f>IF($K$28=0,0,F28/$K$28)</x:f>
+        <x:v>0.46153846153846156</x:v>
+      </x:c>
+      <x:c r="G29" s="565" t="n">
+        <x:f>IF($K$28=0,0,G28/$K$28)</x:f>
+        <x:v>0.02197802197802198</x:v>
+      </x:c>
+      <x:c r="H29" s="565" t="n">
+        <x:f>IF($K$28=0,0,H28/$K$28)</x:f>
+        <x:v>0.04395604395604396</x:v>
+      </x:c>
+      <x:c r="I29" s="565" t="n">
+        <x:f>IF($K$28=0,0,I28/$K$28)</x:f>
+        <x:v>0.15384615384615385</x:v>
+      </x:c>
+      <x:c r="J29" s="565" t="n">
+        <x:f>IF($K$28=0,0,J28/$K$28)</x:f>
+        <x:v>0.054945054945054944</x:v>
+      </x:c>
+      <x:c r="K29" s="565" t="n">
+        <x:f>IF($K$28=0,0,K28/$K$28)</x:f>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="L29" s="84"/>
     </x:row>
@@ -4857,10 +4864,10 @@
         <x:v>남서</x:v>
       </x:c>
       <x:c r="B30" s="109" t="str">
-        <x:v>화성비봉 지역주택조합 아파트 신축공사</x:v>
+        <x:v>남양우미린</x:v>
       </x:c>
       <x:c r="C30" s="109" t="str">
-        <x:v>주식회사 삼진타워</x:v>
+        <x:v>뉴월드타워 주식회사</x:v>
       </x:c>
       <x:c r="D30" s="109"/>
       <x:c r="E30" s="549" t="n">
@@ -4879,10 +4886,10 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="J30" s="546" t="n">
-        <x:v>2</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="K30" s="547" t="n">
-        <x:v>5</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="L30" s="109"/>
     </x:row>
@@ -4891,10 +4898,10 @@
         <x:v>남서</x:v>
       </x:c>
       <x:c r="B31" s="120" t="str">
-        <x:v>오산세교2지구 M1블록 민간임대 주상복합 신축공사</x:v>
+        <x:v>화성비봉 지역주택조합 아파트 신축공사</x:v>
       </x:c>
       <x:c r="C31" s="120" t="str">
-        <x:v>(주)남산공영</x:v>
+        <x:v>주식회사 삼진타워</x:v>
       </x:c>
       <x:c r="D31" s="121"/>
       <x:c r="E31" s="550" t="n">
@@ -4910,13 +4917,13 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="I31" s="550" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="J31" s="550" t="n">
         <x:v>2</x:v>
       </x:c>
       <x:c r="K31" s="548" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="L31" s="120"/>
     </x:row>
@@ -4925,17 +4932,17 @@
         <x:v>남서</x:v>
       </x:c>
       <x:c r="B32" s="151" t="str">
-        <x:v>오산 AMK R&amp;D</x:v>
+        <x:v>오산세교2지구 M1블록 민간임대 주상복합 신축공사</x:v>
       </x:c>
       <x:c r="C32" s="151" t="str">
-        <x:v>신우개발(주)</x:v>
+        <x:v>(주)남산공영</x:v>
       </x:c>
       <x:c r="D32" s="151"/>
       <x:c r="E32" s="551" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="F32" s="551" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="G32" s="551" t="n">
         <x:v>0</x:v>
@@ -4947,11 +4954,10 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="J32" s="551" t="n">
-        <x:v>0</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="K32" s="539" t="n">
-        <x:f>SUM(E32:J32)</x:f>
-        <x:v>1</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="L32" s="119"/>
     </x:row>
@@ -4960,142 +4966,140 @@
         <x:v>남서</x:v>
       </x:c>
       <x:c r="B33" s="153" t="str">
-        <x:v>오산세교우미린레이크시티</x:v>
+        <x:v>오산 AMK R&amp;D</x:v>
       </x:c>
       <x:c r="C33" s="153" t="str">
-        <x:v>뉴월드타워 주식회사</x:v>
+        <x:v>신우개발(주)</x:v>
       </x:c>
       <x:c r="D33" s="153"/>
       <x:c r="E33" s="540" t="n">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="F33" s="540" t="n">
-        <x:v>4</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="G33" s="540" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="H33" s="540" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="I33" s="540" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="J33" s="540" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="K33" s="541" t="n">
-        <x:v>8</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="L33" s="38"/>
     </x:row>
     <x:row r="34" s="14" customFormat="1">
       <x:c r="A34" s="38" t="str">
-        <x:v>남서지부 소계</x:v>
-      </x:c>
-      <x:c r="B34" s="38"/>
-      <x:c r="C34" s="38"/>
+        <x:v>남서</x:v>
+      </x:c>
+      <x:c r="B34" s="38" t="str">
+        <x:v>오산세교우미린레이크시티</x:v>
+      </x:c>
+      <x:c r="C34" s="38" t="str">
+        <x:v>뉴월드타워 주식회사</x:v>
+      </x:c>
       <x:c r="D34" s="38"/>
       <x:c r="E34" s="540" t="n">
-        <x:f>SUM(E29:E33)</x:f>
-        <x:v>6</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="F34" s="540" t="n">
-        <x:f>SUM(F29:F33)</x:f>
-        <x:v>7</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="G34" s="540" t="n">
-        <x:f>SUM(G29:G33)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="H34" s="540" t="n">
-        <x:f>SUM(H29:H33)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="I34" s="540" t="n">
-        <x:f>SUM(I29:I33)</x:f>
-        <x:v>3</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="J34" s="540" t="n">
-        <x:f>SUM(J29:J33)</x:f>
-        <x:v>4</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="K34" s="540" t="n">
-        <x:f>SUM(K29:K33)</x:f>
-        <x:v>21</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="L34" s="38"/>
     </x:row>
     <x:row r="35" s="14" customFormat="1" ht="17.25">
       <x:c r="A35" s="83" t="str">
-        <x:v>소계퍼센테이지</x:v>
+        <x:v>남서지부 소계</x:v>
       </x:c>
       <x:c r="B35" s="84"/>
       <x:c r="C35" s="84"/>
       <x:c r="D35" s="84"/>
-      <x:c r="E35" s="565" t="n">
-        <x:f>IF($K$34=0,0,E34/$K$34)</x:f>
-        <x:v>0.2857142857142857</x:v>
-      </x:c>
-      <x:c r="F35" s="565" t="n">
-        <x:f>IF($K$34=0,0,F34/$K$34)</x:f>
-        <x:v>0.3333333333333333</x:v>
-      </x:c>
-      <x:c r="G35" s="565" t="n">
-        <x:f>IF($K$34=0,0,G34/$K$34)</x:f>
-        <x:v>0.047619047619047616</x:v>
-      </x:c>
-      <x:c r="H35" s="565" t="n">
-        <x:f>IF($K$34=0,0,H34/$K$34)</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="I35" s="565" t="n">
-        <x:f>IF($K$34=0,0,I34/$K$34)</x:f>
-        <x:v>0.14285714285714285</x:v>
-      </x:c>
-      <x:c r="J35" s="565" t="n">
-        <x:f>IF($K$34=0,0,J34/$K$34)</x:f>
-        <x:v>0.19047619047619047</x:v>
-      </x:c>
-      <x:c r="K35" s="565" t="n">
-        <x:f>IF($K$34=0,0,K34/$K$34)</x:f>
-        <x:v>1</x:v>
+      <x:c r="E35" s="545" t="n">
+        <x:f>SUM(E30:E34)</x:f>
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="F35" s="545" t="n">
+        <x:f>SUM(F30:F34)</x:f>
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="G35" s="545" t="n">
+        <x:f>SUM(G30:G34)</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="H35" s="545" t="n">
+        <x:f>SUM(H30:H34)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I35" s="545" t="n">
+        <x:f>SUM(I30:I34)</x:f>
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="J35" s="545" t="n">
+        <x:f>SUM(J30:J34)</x:f>
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="K35" s="545" t="n">
+        <x:f>SUM(K30:K34)</x:f>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="L35" s="84"/>
     </x:row>
     <x:row r="36">
       <x:c r="A36" s="108" t="str">
-        <x:v>동부</x:v>
-      </x:c>
-      <x:c r="B36" s="110" t="str">
-        <x:v>이천한양</x:v>
-      </x:c>
-      <x:c r="C36" s="110" t="str">
-        <x:v>주식회사 현성건설</x:v>
-      </x:c>
-      <x:c r="D36" s="110" t="str">
-        <x:v>현성</x:v>
-      </x:c>
-      <x:c r="E36" s="98" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="F36" s="98" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="G36" s="98" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="H36" s="98" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="I36" s="98" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="J36" s="98" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="K36" s="98" t="n">
-        <x:v>0</x:v>
+        <x:v>소계퍼센테이지</x:v>
+      </x:c>
+      <x:c r="B36" s="110"/>
+      <x:c r="C36" s="110"/>
+      <x:c r="D36" s="110"/>
+      <x:c r="E36" s="565" t="n">
+        <x:f>IF($K$35=0,0,E35/$K$35)</x:f>
+        <x:v>0.2857142857142857</x:v>
+      </x:c>
+      <x:c r="F36" s="565" t="n">
+        <x:f>IF($K$35=0,0,F35/$K$35)</x:f>
+        <x:v>0.3333333333333333</x:v>
+      </x:c>
+      <x:c r="G36" s="565" t="n">
+        <x:f>IF($K$35=0,0,G35/$K$35)</x:f>
+        <x:v>0.047619047619047616</x:v>
+      </x:c>
+      <x:c r="H36" s="565" t="n">
+        <x:f>IF($K$35=0,0,H35/$K$35)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I36" s="565" t="n">
+        <x:f>IF($K$35=0,0,I35/$K$35)</x:f>
+        <x:v>0.14285714285714285</x:v>
+      </x:c>
+      <x:c r="J36" s="565" t="n">
+        <x:f>IF($K$35=0,0,J35/$K$35)</x:f>
+        <x:v>0.19047619047619047</x:v>
+      </x:c>
+      <x:c r="K36" s="565" t="n">
+        <x:f>IF($K$35=0,0,K35/$K$35)</x:f>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="L36" s="110" t="str">
         <x:v>통계제외</x:v>
@@ -5106,17 +5110,19 @@
         <x:v>동부</x:v>
       </x:c>
       <x:c r="B37" s="115" t="str">
-        <x:v>요진건설</x:v>
+        <x:v>이천한양</x:v>
       </x:c>
       <x:c r="C37" s="115" t="str">
-        <x:v>주식회사 한산타워</x:v>
-      </x:c>
-      <x:c r="D37" s="115"/>
+        <x:v>주식회사 현성건설</x:v>
+      </x:c>
+      <x:c r="D37" s="115" t="str">
+        <x:v>현성</x:v>
+      </x:c>
       <x:c r="E37" s="537" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="F37" s="537" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="G37" s="537" t="n">
         <x:v>0</x:v>
@@ -5128,10 +5134,10 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="J37" s="537" t="n">
-        <x:v>0</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="K37" s="548" t="n">
-        <x:v>2</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="L37" s="118"/>
     </x:row>
@@ -5140,10 +5146,10 @@
         <x:v>동부</x:v>
       </x:c>
       <x:c r="B38" s="151" t="str">
-        <x:v>홍문2지구 공동주택</x:v>
+        <x:v>요진건설</x:v>
       </x:c>
       <x:c r="C38" s="151" t="str">
-        <x:v>(주)한진</x:v>
+        <x:v>주식회사 한산타워</x:v>
       </x:c>
       <x:c r="D38" s="151"/>
       <x:c r="E38" s="551" t="n">
@@ -5152,14 +5158,20 @@
       <x:c r="F38" s="551" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="G38" s="551"/>
-      <x:c r="H38" s="551"/>
-      <x:c r="I38" s="551"/>
+      <x:c r="G38" s="551" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H38" s="551" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I38" s="551" t="n">
+        <x:v>0</x:v>
+      </x:c>
       <x:c r="J38" s="551" t="n">
-        <x:v>2</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="K38" s="539" t="n">
-        <x:v>4</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="L38" s="119"/>
     </x:row>
@@ -5168,33 +5180,26 @@
         <x:v>동부</x:v>
       </x:c>
       <x:c r="B39" s="154" t="str">
-        <x:v>이천 증포5지구 칸타빌 에듀파크 신축공사</x:v>
+        <x:v>홍문2지구 공동주택</x:v>
       </x:c>
       <x:c r="C39" s="154" t="str">
-        <x:v>국제산업렌탈(주)</x:v>
+        <x:v>(주)한진</x:v>
       </x:c>
       <x:c r="D39" s="154"/>
       <x:c r="E39" s="542" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="F39" s="542" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="G39" s="542" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="H39" s="542" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="I39" s="542" t="n">
-        <x:v>0</x:v>
-      </x:c>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G39" s="542"/>
+      <x:c r="H39" s="542"/>
+      <x:c r="I39" s="542"/>
       <x:c r="J39" s="542" t="n">
-        <x:v>0</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="K39" s="543" t="n">
-        <x:f>SUM(E39:J39)</x:f>
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="L39" s="82"/>
     </x:row>
@@ -5203,17 +5208,17 @@
         <x:v>동부</x:v>
       </x:c>
       <x:c r="B40" s="43" t="str">
-        <x:v>경안2지구 도시개발사업 주상복합 신축공사</x:v>
+        <x:v>이천 증포5지구 칸타빌 에듀파크 신축공사</x:v>
       </x:c>
       <x:c r="C40" s="43" t="str">
-        <x:v>(주)예림타워</x:v>
+        <x:v>국제산업렌탈(주)</x:v>
       </x:c>
       <x:c r="D40" s="88"/>
       <x:c r="E40" s="542" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="F40" s="542" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="G40" s="542" t="n">
         <x:v>0</x:v>
@@ -5228,115 +5233,115 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="K40" s="543" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="L40" s="82"/>
     </x:row>
     <x:row r="41">
       <x:c r="A41" s="43" t="str">
-        <x:v>동부지부 소계</x:v>
-      </x:c>
-      <x:c r="B41" s="43"/>
-      <x:c r="C41" s="43"/>
+        <x:v>동부</x:v>
+      </x:c>
+      <x:c r="B41" s="43" t="str">
+        <x:v>경안2지구 도시개발사업 주상복합 신축공사</x:v>
+      </x:c>
+      <x:c r="C41" s="43" t="str">
+        <x:v>(주)예림타워</x:v>
+      </x:c>
       <x:c r="D41" s="43"/>
       <x:c r="E41" s="542" t="n">
-        <x:f>SUM(E37:E40)</x:f>
-        <x:v>4</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="F41" s="542" t="n">
-        <x:f>SUM(F37:F40)</x:f>
-        <x:v>5</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="G41" s="542" t="n">
-        <x:f>SUM(G37:G40)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="H41" s="542" t="n">
-        <x:f>SUM(H37:H40)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="I41" s="542" t="n">
-        <x:f>SUM(I37:I40)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="J41" s="542" t="n">
-        <x:f>SUM(J37:J40)</x:f>
-        <x:v>2</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="K41" s="543" t="n">
-        <x:f>SUM(K37:K40)</x:f>
-        <x:v>11</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="L41" s="82"/>
     </x:row>
     <x:row r="42">
       <x:c r="A42" s="43" t="str">
-        <x:v>소계퍼센테이지</x:v>
+        <x:v>동부지부 소계</x:v>
       </x:c>
       <x:c r="B42" s="43"/>
       <x:c r="C42" s="43"/>
       <x:c r="D42" s="43"/>
-      <x:c r="E42" s="102" t="n">
-        <x:f>IF($K$41=0,0,E41/$K$41)</x:f>
-        <x:v>0.36363636363636365</x:v>
-      </x:c>
-      <x:c r="F42" s="102" t="n">
-        <x:f>IF($K$41=0,0,F41/$K$41)</x:f>
-        <x:v>0.45454545454545453</x:v>
-      </x:c>
-      <x:c r="G42" s="102" t="n">
-        <x:f>IF($K$41=0,0,G41/$K$41)</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="H42" s="102" t="n">
-        <x:f>IF($K$41=0,0,H41/$K$41)</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="I42" s="102" t="n">
-        <x:f>IF($K$41=0,0,I41/$K$41)</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="J42" s="102" t="n">
-        <x:f>IF($K$41=0,0,J41/$K$41)</x:f>
-        <x:v>0.18181818181818182</x:v>
-      </x:c>
-      <x:c r="K42" s="103" t="n">
-        <x:f>IF($K$41=0,0,K41/$K$41)</x:f>
-        <x:v>1</x:v>
+      <x:c r="E42" s="542" t="n">
+        <x:f>SUM(E37:E41)</x:f>
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="F42" s="542" t="n">
+        <x:f>SUM(F37:F41)</x:f>
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="G42" s="542" t="n">
+        <x:f>SUM(G37:G41)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H42" s="542" t="n">
+        <x:f>SUM(H37:H41)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I42" s="542" t="n">
+        <x:f>SUM(I37:I41)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J42" s="542" t="n">
+        <x:f>SUM(J37:J41)</x:f>
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="K42" s="543" t="n">
+        <x:f>SUM(K37:K41)</x:f>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="L42" s="82"/>
     </x:row>
     <x:row r="43">
       <x:c r="A43" s="43" t="str">
-        <x:v>서부</x:v>
-      </x:c>
-      <x:c r="B43" s="43" t="str">
-        <x:v>안산프로젝트팀부크(현대건설)</x:v>
-      </x:c>
-      <x:c r="C43" s="43" t="str">
-        <x:v>주식회사 한불타워</x:v>
-      </x:c>
+        <x:v>소계퍼센테이지</x:v>
+      </x:c>
+      <x:c r="B43" s="43"/>
+      <x:c r="C43" s="43"/>
       <x:c r="D43" s="43"/>
-      <x:c r="E43" s="542" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="F43" s="542" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="G43" s="542" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="H43" s="542" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="I43" s="542" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="J43" s="542" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="K43" s="543" t="n">
-        <x:v>2</x:v>
+      <x:c r="E43" s="102" t="n">
+        <x:f>IF($K$42=0,0,E42/$K$42)</x:f>
+        <x:v>0.36363636363636365</x:v>
+      </x:c>
+      <x:c r="F43" s="102" t="n">
+        <x:f>IF($K$42=0,0,F42/$K$42)</x:f>
+        <x:v>0.6363636363636364</x:v>
+      </x:c>
+      <x:c r="G43" s="102" t="n">
+        <x:f>IF($K$42=0,0,G42/$K$42)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H43" s="102" t="n">
+        <x:f>IF($K$42=0,0,H42/$K$42)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I43" s="102" t="n">
+        <x:f>IF($K$42=0,0,I42/$K$42)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J43" s="102" t="n">
+        <x:f>IF($K$42=0,0,J42/$K$42)</x:f>
+        <x:v>0.36363636363636365</x:v>
+      </x:c>
+      <x:c r="K43" s="103" t="n">
+        <x:f>IF($K$42=0,0,K42/$K$42)</x:f>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="L43" s="82"/>
     </x:row>
@@ -5345,10 +5350,10 @@
         <x:v>서부</x:v>
       </x:c>
       <x:c r="B44" s="38" t="str">
-        <x:v>안산글로벌클라우드(삼성물산)</x:v>
+        <x:v>안산프로젝트팀부크(현대건설)</x:v>
       </x:c>
       <x:c r="C44" s="38" t="str">
-        <x:v>정호개발주식회사</x:v>
+        <x:v>주식회사 한불타워</x:v>
       </x:c>
       <x:c r="D44" s="38"/>
       <x:c r="E44" s="540" t="n">
@@ -5379,10 +5384,10 @@
         <x:v>서부</x:v>
       </x:c>
       <x:c r="B45" s="38" t="str">
-        <x:v>하중지구 한신공영</x:v>
+        <x:v>안산글로벌클라우드(삼성물산)</x:v>
       </x:c>
       <x:c r="C45" s="38" t="str">
-        <x:v>(주)신화중공업</x:v>
+        <x:v>정호개발주식회사</x:v>
       </x:c>
       <x:c r="D45" s="38"/>
       <x:c r="E45" s="540" t="n">
@@ -5398,13 +5403,13 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="I45" s="540" t="n">
-        <x:v>2</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="J45" s="540" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="K45" s="540" t="n">
-        <x:v>4</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="L45" s="38"/>
     </x:row>
@@ -5413,17 +5418,17 @@
         <x:v>서부</x:v>
       </x:c>
       <x:c r="B46" s="84" t="str">
-        <x:v>하중지구 양우건설</x:v>
+        <x:v>하중지구 한신공영</x:v>
       </x:c>
       <x:c r="C46" s="84" t="str">
-        <x:v>(주)진성타워</x:v>
+        <x:v>(주)신화중공업</x:v>
       </x:c>
       <x:c r="D46" s="84"/>
       <x:c r="E46" s="545" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="F46" s="545" t="n">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="G46" s="545" t="n">
         <x:v>0</x:v>
@@ -5432,13 +5437,13 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="I46" s="545" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="J46" s="545" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="K46" s="545" t="n">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="L46" s="84"/>
     </x:row>
@@ -5447,14 +5452,14 @@
         <x:v>서부</x:v>
       </x:c>
       <x:c r="B47" s="38" t="str">
-        <x:v>시흥거모지구 S-2BL,B-2BL(대방산업개발)</x:v>
+        <x:v>하중지구 양우건설</x:v>
       </x:c>
       <x:c r="C47" s="38" t="str">
-        <x:v>주식회사 우정타워</x:v>
+        <x:v>(주)진성타워</x:v>
       </x:c>
       <x:c r="D47" s="38"/>
       <x:c r="E47" s="552" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="F47" s="552" t="n">
         <x:v>2</x:v>
@@ -5466,13 +5471,13 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="I47" s="552" t="n">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="J47" s="552" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="K47" s="553" t="n">
-        <x:v>5</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="L47" s="38"/>
     </x:row>
@@ -5481,17 +5486,17 @@
         <x:v>서부</x:v>
       </x:c>
       <x:c r="B48" s="108" t="str">
-        <x:v>배곧서울대학교병원</x:v>
+        <x:v>시흥거모지구 S-2BL,B-2BL(대방산업개발)</x:v>
       </x:c>
       <x:c r="C48" s="108" t="str">
-        <x:v>(주)타워링</x:v>
+        <x:v>주식회사 우정타워</x:v>
       </x:c>
       <x:c r="D48" s="108"/>
       <x:c r="E48" s="545" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="F48" s="545" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="G48" s="545" t="n">
         <x:v>0</x:v>
@@ -5500,13 +5505,13 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="I48" s="545" t="n">
-        <x:v>0</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="J48" s="545" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="K48" s="554" t="n">
-        <x:v>2</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="L48" s="111"/>
     </x:row>
@@ -5515,20 +5520,20 @@
         <x:v>서부</x:v>
       </x:c>
       <x:c r="B49" s="115" t="str">
-        <x:v>시흥하중 A-1BL 공동주택 건설공사</x:v>
+        <x:v>배곧서울대학교병원</x:v>
       </x:c>
       <x:c r="C49" s="115" t="str">
-        <x:v>(주)규람타워렌탈</x:v>
+        <x:v>(주)타워링</x:v>
       </x:c>
       <x:c r="D49" s="121"/>
       <x:c r="E49" s="537" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="F49" s="537" t="n">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="G49" s="537" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="H49" s="537" t="n">
         <x:v>0</x:v>
@@ -5540,7 +5545,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="K49" s="548" t="n">
-        <x:v>4</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="L49" s="118"/>
     </x:row>
@@ -5549,10 +5554,10 @@
         <x:v>서부</x:v>
       </x:c>
       <x:c r="B50" s="151" t="str">
-        <x:v>시흥시 거모지구 B-1블록 공동주택 신축공사</x:v>
+        <x:v>시흥하중 A-1BL 공동주택 건설공사</x:v>
       </x:c>
       <x:c r="C50" s="151" t="str">
-        <x:v>주식회사 필웍스</x:v>
+        <x:v>(주)규람타워렌탈</x:v>
       </x:c>
       <x:c r="D50" s="155"/>
       <x:c r="E50" s="551" t="n">
@@ -5583,10 +5588,10 @@
         <x:v>서부</x:v>
       </x:c>
       <x:c r="B51" s="154" t="str">
-        <x:v>시흥거모 B-6BL 모아엘가&amp;대광로제비앙 공동주택 신축공사</x:v>
+        <x:v>시흥시 거모지구 B-1블록 공동주택 신축공사</x:v>
       </x:c>
       <x:c r="C51" s="154" t="str">
-        <x:v>(주)금강건기</x:v>
+        <x:v>주식회사 필웍스</x:v>
       </x:c>
       <x:c r="D51" s="156"/>
       <x:c r="E51" s="555" t="n">
@@ -5596,13 +5601,13 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G51" s="555" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="H51" s="555" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="I51" s="555" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="J51" s="555" t="n">
         <x:v>0</x:v>
@@ -5617,33 +5622,32 @@
         <x:v>서부</x:v>
       </x:c>
       <x:c r="B52" s="43" t="str">
-        <x:v>시화MTV 지하주차장</x:v>
+        <x:v>시흥거모 B-6BL 모아엘가&amp;대광로제비앙 공동주택 신축공사</x:v>
       </x:c>
       <x:c r="C52" s="43" t="str">
-        <x:v>(주)우리기계산업</x:v>
+        <x:v>(주)금강건기</x:v>
       </x:c>
       <x:c r="D52" s="43"/>
       <x:c r="E52" s="542" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="F52" s="542" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="G52" s="542" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="H52" s="542" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="I52" s="542" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="J52" s="542" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="K52" s="543" t="n">
-        <x:f>SUM(E52:J52)</x:f>
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="L52" s="82" t="str">
         <x:v>원청사: 강산건설(주)</x:v>
@@ -5651,109 +5655,109 @@
     </x:row>
     <x:row r="53">
       <x:c r="A53" s="43" t="str">
-        <x:v>서부지부 소계</x:v>
-      </x:c>
-      <x:c r="B53" s="43"/>
-      <x:c r="C53" s="43"/>
+        <x:v>서부</x:v>
+      </x:c>
+      <x:c r="B53" s="43" t="str">
+        <x:v>시화MTV 지하주차장</x:v>
+      </x:c>
+      <x:c r="C53" s="43" t="str">
+        <x:v>(주)우리기계산업</x:v>
+      </x:c>
       <x:c r="D53" s="43"/>
       <x:c r="E53" s="542" t="n">
-        <x:f>SUM(E43:E52)</x:f>
-        <x:v>9</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="F53" s="542" t="n">
-        <x:f>SUM(F43:F52)</x:f>
-        <x:v>15</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="G53" s="542" t="n">
-        <x:f>SUM(G43:G52)</x:f>
-        <x:v>2</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="H53" s="542" t="n">
-        <x:f>SUM(H43:H52)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="I53" s="542" t="n">
-        <x:f>SUM(I43:I52)</x:f>
-        <x:v>6</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="J53" s="542" t="n">
-        <x:f>SUM(J43:J52)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="K53" s="543" t="n">
-        <x:f>SUM(K43:K52)</x:f>
-        <x:v>33</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="L53" s="82"/>
     </x:row>
     <x:row r="54">
       <x:c r="A54" s="43" t="str">
-        <x:v>소계퍼센테이지</x:v>
+        <x:v>서부지부 소계</x:v>
       </x:c>
       <x:c r="B54" s="43"/>
       <x:c r="C54" s="43"/>
       <x:c r="D54" s="43"/>
-      <x:c r="E54" s="102" t="n">
-        <x:f>IF($K$53=0,0,E53/$K$53)</x:f>
-        <x:v>0.2727272727272727</x:v>
-      </x:c>
-      <x:c r="F54" s="102" t="n">
-        <x:f>IF($K$53=0,0,F53/$K$53)</x:f>
-        <x:v>0.45454545454545453</x:v>
-      </x:c>
-      <x:c r="G54" s="102" t="n">
-        <x:f>IF($K$53=0,0,G53/$K$53)</x:f>
-        <x:v>0.06060606060606061</x:v>
-      </x:c>
-      <x:c r="H54" s="102" t="n">
-        <x:f>IF($K$53=0,0,H53/$K$53)</x:f>
-        <x:v>0.030303030303030304</x:v>
-      </x:c>
-      <x:c r="I54" s="102" t="n">
-        <x:f>IF($K$53=0,0,I53/$K$53)</x:f>
-        <x:v>0.18181818181818182</x:v>
-      </x:c>
-      <x:c r="J54" s="102" t="n">
-        <x:f>IF($K$53=0,0,J53/$K$53)</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="K54" s="103" t="n">
-        <x:f>IF($K$53=0,0,K53/$K$53)</x:f>
-        <x:v>1</x:v>
+      <x:c r="E54" s="542" t="n">
+        <x:f>SUM(E44:E53)</x:f>
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="F54" s="542" t="n">
+        <x:f>SUM(F44:F53)</x:f>
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="G54" s="542" t="n">
+        <x:f>SUM(G44:G53)</x:f>
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="H54" s="542" t="n">
+        <x:f>SUM(H44:H53)</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="I54" s="542" t="n">
+        <x:f>SUM(I44:I53)</x:f>
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="J54" s="542" t="n">
+        <x:f>SUM(J44:J53)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K54" s="543" t="n">
+        <x:f>SUM(K44:K53)</x:f>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="L54" s="82"/>
     </x:row>
     <x:row r="55">
       <x:c r="A55" s="43" t="str">
-        <x:v>북서</x:v>
-      </x:c>
-      <x:c r="B55" s="43" t="str">
-        <x:v>군포시 SGC건설</x:v>
-      </x:c>
-      <x:c r="C55" s="43" t="str">
-        <x:v>(주)한백산업</x:v>
-      </x:c>
+        <x:v>소계퍼센테이지</x:v>
+      </x:c>
+      <x:c r="B55" s="43"/>
+      <x:c r="C55" s="43"/>
       <x:c r="D55" s="43"/>
-      <x:c r="E55" s="542" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="F55" s="542" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="G55" s="542" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="H55" s="542" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="I55" s="542" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="J55" s="542" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="K55" s="543" t="n">
-        <x:v>7</x:v>
+      <x:c r="E55" s="102" t="n">
+        <x:f>IF($K$54=0,0,E54/$K$54)</x:f>
+        <x:v>0.2727272727272727</x:v>
+      </x:c>
+      <x:c r="F55" s="102" t="n">
+        <x:f>IF($K$54=0,0,F54/$K$54)</x:f>
+        <x:v>0.45454545454545453</x:v>
+      </x:c>
+      <x:c r="G55" s="102" t="n">
+        <x:f>IF($K$54=0,0,G54/$K$54)</x:f>
+        <x:v>0.06060606060606061</x:v>
+      </x:c>
+      <x:c r="H55" s="102" t="n">
+        <x:f>IF($K$54=0,0,H54/$K$54)</x:f>
+        <x:v>0.030303030303030304</x:v>
+      </x:c>
+      <x:c r="I55" s="102" t="n">
+        <x:f>IF($K$54=0,0,I54/$K$54)</x:f>
+        <x:v>0.18181818181818182</x:v>
+      </x:c>
+      <x:c r="J55" s="102" t="n">
+        <x:f>IF($K$54=0,0,J54/$K$54)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K55" s="103" t="n">
+        <x:f>IF($K$54=0,0,K54/$K$54)</x:f>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="L55" s="82"/>
     </x:row>
@@ -5762,7 +5766,7 @@
         <x:v>북서</x:v>
       </x:c>
       <x:c r="B56" s="43" t="str">
-        <x:v>관양동 DL이앤씨</x:v>
+        <x:v>군포시 SGC건설</x:v>
       </x:c>
       <x:c r="C56" s="43" t="str">
         <x:v>(주)한백산업</x:v>
@@ -5775,7 +5779,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G56" s="542" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="H56" s="542" t="n">
         <x:v>0</x:v>
@@ -5787,7 +5791,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="K56" s="543" t="n">
-        <x:v>6</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="L56" s="38"/>
     </x:row>
@@ -5799,14 +5803,14 @@
         <x:v>관양동 DL이앤씨</x:v>
       </x:c>
       <x:c r="C57" s="89" t="str">
-        <x:v>벽산중기산업주식회사</x:v>
+        <x:v>(주)한백산업</x:v>
       </x:c>
       <x:c r="D57" s="70"/>
       <x:c r="E57" s="556" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="F57" s="556" t="n">
-        <x:v>1</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="G57" s="556" t="n">
         <x:v>0</x:v>
@@ -5815,13 +5819,13 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="I57" s="556" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="J57" s="556" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="K57" s="556" t="n">
-        <x:v>2</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="L57" s="70"/>
     </x:row>
@@ -5830,10 +5834,10 @@
         <x:v>북서</x:v>
       </x:c>
       <x:c r="B58" s="84" t="str">
-        <x:v>의왕청계 시티건설</x:v>
+        <x:v>관양동 DL이앤씨</x:v>
       </x:c>
       <x:c r="C58" s="84" t="str">
-        <x:v>주식회사 우정타워</x:v>
+        <x:v>벽산중기산업주식회사</x:v>
       </x:c>
       <x:c r="D58" s="84"/>
       <x:c r="E58" s="545" t="n">
@@ -5864,32 +5868,32 @@
         <x:v>북서</x:v>
       </x:c>
       <x:c r="B59" s="38" t="str">
-        <x:v>과천 태왕</x:v>
+        <x:v>의왕청계 시티건설</x:v>
       </x:c>
       <x:c r="C59" s="38" t="str">
-        <x:v>주식회사 비엠케이</x:v>
+        <x:v>주식회사 우정타워</x:v>
       </x:c>
       <x:c r="D59" s="38"/>
       <x:c r="E59" s="552" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="F59" s="552" t="n">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="G59" s="552" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="H59" s="552" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="I59" s="552" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="J59" s="552" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="K59" s="553" t="n">
-        <x:v>6</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="L59" s="38"/>
     </x:row>
@@ -5898,23 +5902,23 @@
         <x:v>북서</x:v>
       </x:c>
       <x:c r="B60" s="108" t="str">
-        <x:v>과천 주암동 디에이치 아델스타(현대건설)</x:v>
+        <x:v>과천 태왕</x:v>
       </x:c>
       <x:c r="C60" s="108" t="str">
-        <x:v>(주)국영타워랜드</x:v>
+        <x:v>주식회사 비엠케이</x:v>
       </x:c>
       <x:c r="D60" s="108"/>
       <x:c r="E60" s="545" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="F60" s="545" t="n">
-        <x:v>3</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="G60" s="545" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="H60" s="545" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="I60" s="545" t="n">
         <x:v>1</x:v>
@@ -5923,7 +5927,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="K60" s="554" t="n">
-        <x:v>5</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="L60" s="111"/>
     </x:row>
@@ -5932,17 +5936,17 @@
         <x:v>북서</x:v>
       </x:c>
       <x:c r="B61" s="115" t="str">
-        <x:v>안양 샘병원</x:v>
+        <x:v>과천 주암동 디에이치 아델스타(현대건설)</x:v>
       </x:c>
       <x:c r="C61" s="115" t="str">
-        <x:v>주식회사 가람타워</x:v>
+        <x:v>(주)국영타워랜드</x:v>
       </x:c>
       <x:c r="D61" s="115"/>
       <x:c r="E61" s="537" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="F61" s="537" t="n">
-        <x:v>0</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="G61" s="537" t="n">
         <x:v>0</x:v>
@@ -5951,13 +5955,13 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="I61" s="537" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="J61" s="537" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="K61" s="548" t="n">
-        <x:v>1</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="L61" s="118"/>
     </x:row>
@@ -5966,17 +5970,17 @@
         <x:v>북서</x:v>
       </x:c>
       <x:c r="B62" s="151" t="str">
-        <x:v>안양 박달동 신안아파트 재건축(현대산업개발)</x:v>
+        <x:v>안양 샘병원</x:v>
       </x:c>
       <x:c r="C62" s="151" t="str">
-        <x:v>주식회사 비엠케이</x:v>
+        <x:v>주식회사 가람타워</x:v>
       </x:c>
       <x:c r="D62" s="151"/>
       <x:c r="E62" s="551" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="F62" s="551" t="n">
-        <x:v>2</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="G62" s="551" t="n">
         <x:v>0</x:v>
@@ -5985,13 +5989,13 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="I62" s="551" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="J62" s="551" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="K62" s="539" t="n">
-        <x:v>4</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="L62" s="119"/>
     </x:row>
@@ -6000,10 +6004,10 @@
         <x:v>북서</x:v>
       </x:c>
       <x:c r="B63" s="157" t="str">
-        <x:v>안양역세권지구 재개발정비사업(현대산업개발)</x:v>
+        <x:v>안양 박달동 신안아파트 재건축(현대산업개발)</x:v>
       </x:c>
       <x:c r="C63" s="157" t="str">
-        <x:v>오투기계산업(주)</x:v>
+        <x:v>주식회사 비엠케이</x:v>
       </x:c>
       <x:c r="D63" s="156"/>
       <x:c r="E63" s="555" t="n">
@@ -6034,17 +6038,17 @@
         <x:v>북서</x:v>
       </x:c>
       <x:c r="B64" s="43" t="str">
-        <x:v>관양동 오피스텔 신축공사</x:v>
+        <x:v>안양역세권지구 재개발정비사업(현대산업개발)</x:v>
       </x:c>
       <x:c r="C64" s="43" t="str">
-        <x:v>(주)유건설 (단종계약)</x:v>
+        <x:v>오투기계산업(주)</x:v>
       </x:c>
       <x:c r="D64" s="88"/>
       <x:c r="E64" s="542" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="F64" s="542" t="n">
-        <x:v>0</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="G64" s="542" t="n">
         <x:v>0</x:v>
@@ -6053,122 +6057,121 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="I64" s="542" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="J64" s="542" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="K64" s="543" t="n">
-        <x:f>SUM(E64:J64)</x:f>
-        <x:v>1</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="L64" s="82"/>
     </x:row>
     <x:row r="65">
       <x:c r="A65" s="43" t="str">
-        <x:v>북서지부 소계</x:v>
-      </x:c>
-      <x:c r="B65" s="43"/>
-      <x:c r="C65" s="43"/>
+        <x:v>북서</x:v>
+      </x:c>
+      <x:c r="B65" s="43" t="str">
+        <x:v>관양동 오피스텔 신축공사</x:v>
+      </x:c>
+      <x:c r="C65" s="43" t="str">
+        <x:v>(주)유건설 (단종계약)</x:v>
+      </x:c>
       <x:c r="D65" s="43"/>
       <x:c r="E65" s="542" t="n">
-        <x:f>SUM(E55:E64)</x:f>
-        <x:v>12</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="F65" s="542" t="n">
-        <x:f>SUM(F55:F64)</x:f>
-        <x:v>17</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="G65" s="542" t="n">
-        <x:f>SUM(G55:G64)</x:f>
-        <x:v>2</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="H65" s="542" t="n">
-        <x:f>SUM(H55:H64)</x:f>
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="I65" s="542" t="n">
-        <x:f>SUM(I55:I64)</x:f>
-        <x:v>6</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="J65" s="542" t="n">
-        <x:f>SUM(J55:J64)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="K65" s="543" t="n">
-        <x:f>SUM(K55:K64)</x:f>
-        <x:v>38</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="L65" s="82"/>
     </x:row>
     <x:row r="66" s="14" customFormat="1" ht="17.25">
       <x:c r="A66" s="43" t="str">
-        <x:v>소계퍼센테이지</x:v>
+        <x:v>북서지부 소계</x:v>
       </x:c>
       <x:c r="B66" s="43"/>
       <x:c r="C66" s="43"/>
       <x:c r="D66" s="43"/>
-      <x:c r="E66" s="102" t="n">
-        <x:f>IF($K$65=0,0,E65/$K$65)</x:f>
-        <x:v>0.3157894736842105</x:v>
-      </x:c>
-      <x:c r="F66" s="102" t="n">
-        <x:f>IF($K$65=0,0,F65/$K$65)</x:f>
-        <x:v>0.4473684210526316</x:v>
-      </x:c>
-      <x:c r="G66" s="102" t="n">
-        <x:f>IF($K$65=0,0,G65/$K$65)</x:f>
-        <x:v>0.05263157894736842</x:v>
-      </x:c>
-      <x:c r="H66" s="102" t="n">
-        <x:f>IF($K$65=0,0,H65/$K$65)</x:f>
-        <x:v>0.02631578947368421</x:v>
-      </x:c>
-      <x:c r="I66" s="102" t="n">
-        <x:f>IF($K$65=0,0,I65/$K$65)</x:f>
-        <x:v>0.15789473684210525</x:v>
-      </x:c>
-      <x:c r="J66" s="102" t="n">
-        <x:f>IF($K$65=0,0,J65/$K$65)</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="K66" s="103" t="n">
-        <x:f>IF($K$65=0,0,K65/$K$65)</x:f>
-        <x:v>1</x:v>
+      <x:c r="E66" s="542" t="n">
+        <x:f>SUM(E56:E65)</x:f>
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="F66" s="542" t="n">
+        <x:f>SUM(F56:F65)</x:f>
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="G66" s="542" t="n">
+        <x:f>SUM(G56:G65)</x:f>
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="H66" s="542" t="n">
+        <x:f>SUM(H56:H65)</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="I66" s="542" t="n">
+        <x:f>SUM(I56:I65)</x:f>
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="J66" s="542" t="n">
+        <x:f>SUM(J56:J65)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K66" s="543" t="n">
+        <x:f>SUM(K56:K65)</x:f>
+        <x:v>38</x:v>
       </x:c>
       <x:c r="L66" s="38"/>
     </x:row>
     <x:row r="67" s="14" customFormat="1" ht="17.25">
       <x:c r="A67" s="43" t="str">
-        <x:v>용인</x:v>
-      </x:c>
-      <x:c r="B67" s="43" t="str">
-        <x:v>양지 대우 원클러스터</x:v>
-      </x:c>
-      <x:c r="C67" s="43" t="str">
-        <x:v>(주)규람타워렌탈</x:v>
-      </x:c>
+        <x:v>소계퍼센테이지</x:v>
+      </x:c>
+      <x:c r="B67" s="43"/>
+      <x:c r="C67" s="43"/>
       <x:c r="D67" s="43"/>
-      <x:c r="E67" s="542" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="F67" s="542" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="G67" s="542" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="H67" s="542" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="I67" s="542" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="J67" s="542" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="K67" s="543" t="n">
-        <x:v>4</x:v>
+      <x:c r="E67" s="102" t="n">
+        <x:f>IF($K$66=0,0,E66/$K$66)</x:f>
+        <x:v>0.3157894736842105</x:v>
+      </x:c>
+      <x:c r="F67" s="102" t="n">
+        <x:f>IF($K$66=0,0,F66/$K$66)</x:f>
+        <x:v>0.4473684210526316</x:v>
+      </x:c>
+      <x:c r="G67" s="102" t="n">
+        <x:f>IF($K$66=0,0,G66/$K$66)</x:f>
+        <x:v>0.05263157894736842</x:v>
+      </x:c>
+      <x:c r="H67" s="102" t="n">
+        <x:f>IF($K$66=0,0,H66/$K$66)</x:f>
+        <x:v>0.02631578947368421</x:v>
+      </x:c>
+      <x:c r="I67" s="102" t="n">
+        <x:f>IF($K$66=0,0,I66/$K$66)</x:f>
+        <x:v>0.15789473684210525</x:v>
+      </x:c>
+      <x:c r="J67" s="102" t="n">
+        <x:f>IF($K$66=0,0,J66/$K$66)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K67" s="103" t="n">
+        <x:f>IF($K$66=0,0,K66/$K$66)</x:f>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="L67" s="38"/>
     </x:row>
@@ -6177,26 +6180,26 @@
         <x:v>용인</x:v>
       </x:c>
       <x:c r="B68" s="43" t="str">
-        <x:v>양지 SM경남 아너스빌</x:v>
+        <x:v>양지 대우 원클러스터</x:v>
       </x:c>
       <x:c r="C68" s="43" t="str">
-        <x:v>주식회사 비엠케이</x:v>
+        <x:v>(주)규람타워렌탈</x:v>
       </x:c>
       <x:c r="D68" s="43"/>
       <x:c r="E68" s="542" t="n">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="F68" s="542" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="G68" s="542" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="H68" s="542" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="I68" s="542" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="J68" s="542" t="n">
         <x:v>0</x:v>
@@ -6211,26 +6214,26 @@
         <x:v>용인</x:v>
       </x:c>
       <x:c r="B69" s="38" t="str">
-        <x:v>역북 푸르지오 클루센트(대우건설)</x:v>
+        <x:v>양지 SM경남 아너스빌</x:v>
       </x:c>
       <x:c r="C69" s="38" t="str">
-        <x:v>벽산중기산업주식회사</x:v>
+        <x:v>주식회사 비엠케이</x:v>
       </x:c>
       <x:c r="D69" s="38"/>
       <x:c r="E69" s="540" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="F69" s="540" t="n">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="G69" s="540" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="H69" s="540" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="I69" s="540" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="J69" s="540" t="n">
         <x:v>0</x:v>
@@ -6245,25 +6248,23 @@
         <x:v>용인</x:v>
       </x:c>
       <x:c r="B70" s="90" t="str">
-        <x:v>고림 대광로제비앙</x:v>
+        <x:v>역북 푸르지오 클루센트(대우건설)</x:v>
       </x:c>
       <x:c r="C70" s="90" t="str">
-        <x:v>주식회사 현성건설</x:v>
-      </x:c>
-      <x:c r="D70" s="90" t="str">
-        <x:v>현성</x:v>
-      </x:c>
+        <x:v>벽산중기산업주식회사</x:v>
+      </x:c>
+      <x:c r="D70" s="90"/>
       <x:c r="E70" s="557" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="F70" s="557" t="n">
-        <x:v>3</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="G70" s="557" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="H70" s="557" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="I70" s="557" t="n">
         <x:v>1</x:v>
@@ -6272,7 +6273,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="K70" s="557" t="n">
-        <x:v>0</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="L70" s="90" t="str">
         <x:v>통계제외</x:v>
@@ -6283,17 +6284,19 @@
         <x:v>용인</x:v>
       </x:c>
       <x:c r="B71" s="69" t="str">
-        <x:v>백암 오뚜기물류센타</x:v>
+        <x:v>고림 대광로제비앙</x:v>
       </x:c>
       <x:c r="C71" s="69" t="str">
-        <x:v>주식회사 가람타워</x:v>
-      </x:c>
-      <x:c r="D71" s="69"/>
+        <x:v>주식회사 현성건설</x:v>
+      </x:c>
+      <x:c r="D71" s="69" t="str">
+        <x:v>현성</x:v>
+      </x:c>
       <x:c r="E71" s="534" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F71" s="534" t="n">
-        <x:v>1</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="G71" s="534" t="n">
         <x:v>0</x:v>
@@ -6302,13 +6305,13 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I71" s="534" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="J71" s="534" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="K71" s="534" t="n">
-        <x:v>2</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="L71" s="69"/>
     </x:row>
@@ -6317,10 +6320,10 @@
         <x:v>용인</x:v>
       </x:c>
       <x:c r="B72" s="91" t="str">
-        <x:v>마평동 여성복지회관</x:v>
+        <x:v>백암 오뚜기물류센타</x:v>
       </x:c>
       <x:c r="C72" s="91" t="str">
-        <x:v>(주)무기타워렌탈</x:v>
+        <x:v>주식회사 가람타워</x:v>
       </x:c>
       <x:c r="D72" s="91"/>
       <x:c r="E72" s="544" t="n">
@@ -6333,7 +6336,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="H72" s="544" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="I72" s="544" t="n">
         <x:v>0</x:v>
@@ -6342,7 +6345,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="K72" s="544" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="L72" s="92"/>
     </x:row>
@@ -6351,14 +6354,14 @@
         <x:v>용인</x:v>
       </x:c>
       <x:c r="B73" s="93" t="str">
-        <x:v>용인 라온프라이빗</x:v>
+        <x:v>마평동 여성복지회관</x:v>
       </x:c>
       <x:c r="C73" s="93" t="str">
-        <x:v>(주)우성건설기계</x:v>
+        <x:v>(주)무기타워렌탈</x:v>
       </x:c>
       <x:c r="D73" s="93"/>
       <x:c r="E73" s="558" t="n">
-        <x:v>2</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="F73" s="558" t="n">
         <x:v>1</x:v>
@@ -6376,7 +6379,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="K73" s="558" t="n">
-        <x:v>3</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="L73" s="94"/>
     </x:row>
@@ -6385,20 +6388,20 @@
         <x:v>용인</x:v>
       </x:c>
       <x:c r="B74" s="112" t="str">
-        <x:v>용인덕성 AI데이터센터 신축공사</x:v>
+        <x:v>용인 라온프라이빗</x:v>
       </x:c>
       <x:c r="C74" s="112" t="str">
-        <x:v>(주)타워랜드</x:v>
+        <x:v>(주)우성건설기계</x:v>
       </x:c>
       <x:c r="D74" s="112"/>
       <x:c r="E74" s="559" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="F74" s="559" t="n">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="G74" s="559" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="H74" s="559" t="n">
         <x:v>0</x:v>
@@ -6410,7 +6413,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="K74" s="559" t="n">
-        <x:v>4</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="L74" s="113"/>
     </x:row>
@@ -6419,34 +6422,32 @@
         <x:v>용인</x:v>
       </x:c>
       <x:c r="B75" s="122" t="str">
-        <x:v>용인클러스터 상생협력시설(기숙사 1차)</x:v>
+        <x:v>용인덕성 AI데이터센터 신축공사</x:v>
       </x:c>
       <x:c r="C75" s="122" t="str">
-        <x:v>(주)규람타워렌탈</x:v>
-      </x:c>
-      <x:c r="D75" s="122" t="str">
-        <x:v>원철규(미정3)</x:v>
-      </x:c>
+        <x:v>(주)타워랜드</x:v>
+      </x:c>
+      <x:c r="D75" s="122"/>
       <x:c r="E75" s="560" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="F75" s="560" t="n">
-        <x:v>0</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="G75" s="560" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="H75" s="560" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="I75" s="560" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="J75" s="560" t="n">
-        <x:v>3</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="K75" s="560" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="L75" s="123"/>
     </x:row>
@@ -6455,17 +6456,19 @@
         <x:v>용인</x:v>
       </x:c>
       <x:c r="B76" s="158" t="str">
-        <x:v>수지자이에디시온</x:v>
+        <x:v>용인클러스터 상생협력시설(기숙사 1차)</x:v>
       </x:c>
       <x:c r="C76" s="158" t="str">
-        <x:v>(주)한진</x:v>
-      </x:c>
-      <x:c r="D76" s="158"/>
+        <x:v>(주)규람타워렌탈</x:v>
+      </x:c>
+      <x:c r="D76" s="158" t="str">
+        <x:v>원철규(미정3)</x:v>
+      </x:c>
       <x:c r="E76" s="561" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="F76" s="561" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="G76" s="561" t="n">
         <x:v>0</x:v>
@@ -6477,10 +6480,10 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="J76" s="561" t="n">
-        <x:v>0</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="K76" s="561" t="n">
-        <x:v>3</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="L76" s="124"/>
     </x:row>
@@ -6489,17 +6492,17 @@
         <x:v>용인</x:v>
       </x:c>
       <x:c r="B77" s="160" t="str">
-        <x:v>기흥변전소</x:v>
+        <x:v>수지자이에디시온</x:v>
       </x:c>
       <x:c r="C77" s="160" t="str">
-        <x:v>(주)대원타워렌탈</x:v>
+        <x:v>(주)한진</x:v>
       </x:c>
       <x:c r="D77" s="160"/>
       <x:c r="E77" s="555" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="F77" s="555" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="G77" s="555" t="n">
         <x:v>0</x:v>
@@ -6514,7 +6517,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="K77" s="561" t="n">
-        <x:v>1</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="L77" s="90"/>
     </x:row>
@@ -6523,10 +6526,10 @@
         <x:v>용인</x:v>
       </x:c>
       <x:c r="B78" s="69" t="str">
-        <x:v>한양립스</x:v>
+        <x:v>기흥변전소</x:v>
       </x:c>
       <x:c r="C78" s="69" t="str">
-        <x:v>(주)제이에스글로벌산업</x:v>
+        <x:v>(주)대원타워렌탈</x:v>
       </x:c>
       <x:c r="D78" s="69"/>
       <x:c r="E78" s="534" t="n">
@@ -6539,7 +6542,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="H78" s="534" t="n">
-        <x:v>2</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="I78" s="534" t="n">
         <x:v>1</x:v>
@@ -6548,8 +6551,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="K78" s="534" t="n">
-        <x:f>SUM(E78:J78)</x:f>
-        <x:v>3</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="L78" s="69"/>
     </x:row>
@@ -6558,35 +6560,32 @@
         <x:v>용인</x:v>
       </x:c>
       <x:c r="B79" s="91" t="str">
-        <x:v>신광교 클라우드 시티 신축공사</x:v>
+        <x:v>한양립스</x:v>
       </x:c>
       <x:c r="C79" s="91" t="str">
-        <x:v>(주)성광엔지니어링</x:v>
-      </x:c>
-      <x:c r="D79" s="91" t="str">
-        <x:v>원청사: 현대엔지니어링(주)</x:v>
-      </x:c>
+        <x:v>(주)제이에스글로벌산업</x:v>
+      </x:c>
+      <x:c r="D79" s="91"/>
       <x:c r="E79" s="544" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="F79" s="544" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="G79" s="544" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="H79" s="544" t="n">
-        <x:v>0</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="I79" s="544" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="J79" s="544" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K79" s="544" t="n">
         <x:v>3</x:v>
-      </x:c>
-      <x:c r="K79" s="544" t="n">
-        <x:f>SUM(E79:J79)</x:f>
-        <x:v>5</x:v>
       </x:c>
       <x:c r="L79" s="91" t="str">
         <x:v>2026-10-17 입사 / 현장명 정정 / 총 1→5대 (2026-10-19 명단)</x:v>
@@ -6594,109 +6593,111 @@
     </x:row>
     <x:row r="80">
       <x:c r="A80" s="93" t="str">
-        <x:v>용인지부 소계</x:v>
-      </x:c>
-      <x:c r="B80" s="93"/>
-      <x:c r="C80" s="93"/>
-      <x:c r="D80" s="93"/>
+        <x:v>용인</x:v>
+      </x:c>
+      <x:c r="B80" s="93" t="str">
+        <x:v>신광교 클라우드 시티 신축공사</x:v>
+      </x:c>
+      <x:c r="C80" s="93" t="str">
+        <x:v>(주)성광엔지니어링</x:v>
+      </x:c>
+      <x:c r="D80" s="93" t="str">
+        <x:v>원청사: 현대엔지니어링(주)</x:v>
+      </x:c>
       <x:c r="E80" s="558" t="n">
-        <x:f>SUM(E67:E69,E71:E79)</x:f>
-        <x:v>10</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="F80" s="558" t="n">
-        <x:f>SUM(F67:F69,F71:F79)</x:f>
-        <x:v>12</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="G80" s="558" t="n">
-        <x:f>SUM(G67:G69,G71:G79)</x:f>
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="H80" s="558" t="n">
-        <x:f>SUM(H67:H69,H71:H79)</x:f>
-        <x:v>4</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="I80" s="558" t="n">
-        <x:f>SUM(I67:I69,I71:I79)</x:f>
-        <x:v>6</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="J80" s="558" t="n">
-        <x:f>SUM(J67:J69,J71:J79)</x:f>
-        <x:v>6</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="K80" s="558" t="n">
-        <x:f>SUM(K67:K69,K71:K79)</x:f>
-        <x:v>39</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="L80" s="93"/>
     </x:row>
     <x:row r="81">
       <x:c r="A81" s="114" t="str">
-        <x:v>소계퍼센테이지</x:v>
+        <x:v>용인지부 소계</x:v>
       </x:c>
       <x:c r="B81" s="114"/>
       <x:c r="C81" s="114"/>
       <x:c r="D81" s="114"/>
-      <x:c r="E81" s="566" t="n">
-        <x:f>IF($K$80=0,0,E80/$K$80)</x:f>
-        <x:v>0.2564102564102564</x:v>
-      </x:c>
-      <x:c r="F81" s="566" t="n">
-        <x:f>IF($K$80=0,0,F80/$K$80)</x:f>
-        <x:v>0.3076923076923077</x:v>
-      </x:c>
-      <x:c r="G81" s="566" t="n">
-        <x:f>IF($K$80=0,0,G80/$K$80)</x:f>
-        <x:v>0.02564102564102564</x:v>
-      </x:c>
-      <x:c r="H81" s="566" t="n">
-        <x:f>IF($K$80=0,0,H80/$K$80)</x:f>
-        <x:v>0.10256410256410256</x:v>
-      </x:c>
-      <x:c r="I81" s="566" t="n">
-        <x:f>IF($K$80=0,0,I80/$K$80)</x:f>
-        <x:v>0.15384615384615385</x:v>
-      </x:c>
-      <x:c r="J81" s="566" t="n">
-        <x:f>IF($K$80=0,0,J80/$K$80)</x:f>
-        <x:v>0.15384615384615385</x:v>
-      </x:c>
-      <x:c r="K81" s="566" t="n">
-        <x:f>IF($K$80=0,0,K80/$K$80)</x:f>
-        <x:v>1</x:v>
+      <x:c r="E81" s="568" t="n">
+        <x:f>SUM(E68:E80)</x:f>
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F81" s="568" t="n">
+        <x:f>SUM(F68:F80)</x:f>
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="G81" s="568" t="n">
+        <x:f>SUM(G68:G80)</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="H81" s="568" t="n">
+        <x:f>SUM(H68:H80)</x:f>
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="I81" s="568" t="n">
+        <x:f>SUM(I68:I80)</x:f>
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="J81" s="568" t="n">
+        <x:f>SUM(J68:J80)</x:f>
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="K81" s="568" t="n">
+        <x:f>SUM(K68:K80)</x:f>
+        <x:v>39</x:v>
       </x:c>
       <x:c r="L81" s="114"/>
     </x:row>
     <x:row r="82">
       <x:c r="A82" s="125" t="str">
-        <x:v>중부</x:v>
-      </x:c>
-      <x:c r="B82" s="125" t="str">
-        <x:v>당수동 한신</x:v>
-      </x:c>
-      <x:c r="C82" s="125" t="str">
-        <x:v>주식회사월드타워</x:v>
-      </x:c>
+        <x:v>소계퍼센테이지</x:v>
+      </x:c>
+      <x:c r="B82" s="125"/>
+      <x:c r="C82" s="125"/>
       <x:c r="D82" s="125"/>
-      <x:c r="E82" s="562" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="F82" s="562" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="G82" s="562" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="H82" s="562" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="I82" s="562" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="J82" s="562" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="K82" s="562" t="n">
-        <x:v>5</x:v>
+      <x:c r="E82" s="569" t="n">
+        <x:f>IF($K$81=0,0,E81/$K$81)</x:f>
+        <x:v>0.2564102564102564</x:v>
+      </x:c>
+      <x:c r="F82" s="569" t="n">
+        <x:f>IF($K$81=0,0,F81/$K$81)</x:f>
+        <x:v>0.38461538461538464</x:v>
+      </x:c>
+      <x:c r="G82" s="569" t="n">
+        <x:f>IF($K$81=0,0,G81/$K$81)</x:f>
+        <x:v>0.02564102564102564</x:v>
+      </x:c>
+      <x:c r="H82" s="569" t="n">
+        <x:f>IF($K$81=0,0,H81/$K$81)</x:f>
+        <x:v>0.1282051282051282</x:v>
+      </x:c>
+      <x:c r="I82" s="569" t="n">
+        <x:f>IF($K$81=0,0,I81/$K$81)</x:f>
+        <x:v>0.1794871794871795</x:v>
+      </x:c>
+      <x:c r="J82" s="569" t="n">
+        <x:f>IF($K$81=0,0,J81/$K$81)</x:f>
+        <x:v>0.15384615384615385</x:v>
+      </x:c>
+      <x:c r="K82" s="569" t="n">
+        <x:f>IF($K$81=0,0,K81/$K$81)</x:f>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="L82" s="125"/>
     </x:row>
@@ -6705,10 +6706,10 @@
         <x:v>중부</x:v>
       </x:c>
       <x:c r="B83" s="161" t="str">
-        <x:v>당수동 한라</x:v>
+        <x:v>당수동 한신</x:v>
       </x:c>
       <x:c r="C83" s="161" t="str">
-        <x:v>벽산중기산업주식회사</x:v>
+        <x:v>주식회사월드타워</x:v>
       </x:c>
       <x:c r="D83" s="161"/>
       <x:c r="E83" s="563" t="n">
@@ -6718,19 +6719,19 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G83" s="563" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="H83" s="563" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="I83" s="563" t="n">
-        <x:v>0</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="J83" s="563" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="K83" s="563" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="L83" s="126"/>
     </x:row>
@@ -6739,26 +6740,26 @@
         <x:v>중부</x:v>
       </x:c>
       <x:c r="B84" s="163" t="str">
-        <x:v>당수동 계룡</x:v>
+        <x:v>당수동 한라</x:v>
       </x:c>
       <x:c r="C84" s="163" t="str">
-        <x:v>주식회사 화성건기</x:v>
+        <x:v>벽산중기산업주식회사</x:v>
       </x:c>
       <x:c r="D84" s="163"/>
       <x:c r="E84" s="555" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="F84" s="555" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="G84" s="555" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="H84" s="555" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="I84" s="555" t="n">
-        <x:v>2</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="J84" s="555" t="n">
         <x:v>0</x:v>
@@ -6773,10 +6774,10 @@
         <x:v>중부</x:v>
       </x:c>
       <x:c r="B85" t="str">
-        <x:v>영화동 두산</x:v>
+        <x:v>당수동 계룡</x:v>
       </x:c>
       <x:c r="C85" t="str">
-        <x:v>(주)야후건기</x:v>
+        <x:v>주식회사 화성건기</x:v>
       </x:c>
       <x:c r="D85"/>
       <x:c r="E85" s="536" t="n">
@@ -6792,13 +6793,13 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="I85" s="536" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="J85" s="536" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="K85" s="536" t="n">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="L85"/>
     </x:row>
@@ -6807,17 +6808,17 @@
         <x:v>중부</x:v>
       </x:c>
       <x:c r="B86" t="str">
-        <x:v>수원 친환경 에너지 개선공사 주기기 구매</x:v>
+        <x:v>영화동 두산</x:v>
       </x:c>
       <x:c r="C86" t="str">
-        <x:v>신우개발(주)</x:v>
+        <x:v>(주)야후건기</x:v>
       </x:c>
       <x:c r="D86"/>
       <x:c r="E86" s="536" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="F86" s="536" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="G86" s="536" t="n">
         <x:v>0</x:v>
@@ -6826,90 +6827,122 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="I86" s="536" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="J86" s="536" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="K86" s="536" t="n">
-        <x:f>SUM(E86:J86)</x:f>
-        <x:v>1</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="L86"/>
     </x:row>
     <x:row r="87">
       <x:c r="A87" t="str">
-        <x:v>중부지부 소계</x:v>
-      </x:c>
-      <x:c r="B87"/>
-      <x:c r="C87"/>
+        <x:v>중부</x:v>
+      </x:c>
+      <x:c r="B87" t="str">
+        <x:v>수원 친환경 에너지 개선공사 주기기 구매</x:v>
+      </x:c>
+      <x:c r="C87" t="str">
+        <x:v>신우개발(주)</x:v>
+      </x:c>
       <x:c r="D87"/>
       <x:c r="E87" s="536" t="n">
-        <x:f>SUM(E82:E86)</x:f>
-        <x:v>5</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="F87" s="536" t="n">
-        <x:f>SUM(F82:F86)</x:f>
-        <x:v>6</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="G87" s="536" t="n">
-        <x:f>SUM(G82:G86)</x:f>
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="H87" s="536" t="n">
-        <x:f>SUM(H82:H86)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="I87" s="536" t="n">
-        <x:f>SUM(I82:I86)</x:f>
-        <x:v>5</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="J87" s="536" t="n">
-        <x:f>SUM(J82:J86)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="K87" s="536" t="n">
-        <x:f>SUM(K82:K86)</x:f>
-        <x:v>17</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="L87"/>
     </x:row>
     <x:row r="88">
       <x:c r="A88" t="str">
-        <x:v>소계퍼센테이지</x:v>
+        <x:v>중부지부 소계</x:v>
       </x:c>
       <x:c r="B88"/>
       <x:c r="C88"/>
       <x:c r="D88"/>
-      <x:c r="E88" s="95" t="n">
-        <x:f>IF($K$87=0,0,E87/$K$87)</x:f>
+      <x:c r="E88" s="536" t="n">
+        <x:f>SUM(E83:E87)</x:f>
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="F88" s="536" t="n">
+        <x:f>SUM(F83:F87)</x:f>
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="G88" s="536" t="n">
+        <x:f>SUM(G83:G87)</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="H88" s="536" t="n">
+        <x:f>SUM(H83:H87)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I88" s="536" t="n">
+        <x:f>SUM(I83:I87)</x:f>
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="J88" s="536" t="n">
+        <x:f>SUM(J83:J87)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K88" s="536" t="n">
+        <x:f>SUM(K83:K87)</x:f>
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="L88"/>
+    </x:row>
+    <x:row r="89">
+      <x:c r="A89" t="str">
+        <x:v>소계퍼센테이지</x:v>
+      </x:c>
+      <x:c r="B89"/>
+      <x:c r="C89"/>
+      <x:c r="D89"/>
+      <x:c r="E89" s="95" t="n">
+        <x:f>IF($K$88=0,0,E88/$K$88)</x:f>
         <x:v>0.29411764705882354</x:v>
       </x:c>
-      <x:c r="F88" s="95" t="n">
-        <x:f>IF($K$87=0,0,F87/$K$87)</x:f>
+      <x:c r="F89" s="95" t="n">
+        <x:f>IF($K$88=0,0,F88/$K$88)</x:f>
         <x:v>0.35294117647058826</x:v>
       </x:c>
-      <x:c r="G88" s="95" t="n">
-        <x:f>IF($K$87=0,0,G87/$K$87)</x:f>
+      <x:c r="G89" s="95" t="n">
+        <x:f>IF($K$88=0,0,G88/$K$88)</x:f>
         <x:v>0.058823529411764705</x:v>
       </x:c>
-      <x:c r="H88" s="95" t="n">
-        <x:f>IF($K$87=0,0,H87/$K$87)</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="I88" s="95" t="n">
-        <x:f>IF($K$87=0,0,I87/$K$87)</x:f>
+      <x:c r="H89" s="95" t="n">
+        <x:f>IF($K$88=0,0,H88/$K$88)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I89" s="95" t="n">
+        <x:f>IF($K$88=0,0,I88/$K$88)</x:f>
         <x:v>0.29411764705882354</x:v>
       </x:c>
-      <x:c r="J88" s="95" t="n">
-        <x:f>IF($K$87=0,0,J87/$K$87)</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="K88" s="95" t="n">
-        <x:f>IF($K$87=0,0,K87/$K$87)</x:f>
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="L88"/>
+      <x:c r="J89" s="95" t="n">
+        <x:f>IF($K$88=0,0,J88/$K$88)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K89" s="95" t="n">
+        <x:f>IF($K$88=0,0,K88/$K$88)</x:f>
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -7338,32 +7371,33 @@
       <x:c r="A14" s="12" t="s">
         <x:v>68</x:v>
       </x:c>
-      <x:c r="B14" s="11">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="C14" s="11">
-        <x:v>3</x:v>
+      <x:c r="B14" s="11" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="C14" s="11" t="n">
+        <x:v>4</x:v>
       </x:c>
       <x:c r="D14" s="11" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="E14" s="11" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="F14" s="11">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G14" s="11">
+      <x:c r="F14" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G14" s="11" t="n">
         <x:v>2</x:v>
       </x:c>
       <x:c r="H14" s="11" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="I14" s="9">
-        <x:v>13</x:v>
-      </x:c>
-      <x:c r="J14" s="34">
-        <x:v>0.23076923076923081</x:v>
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="I14" s="9" t="n">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="J14" s="34" t="n">
+        <x:f>IF(I14=0,0,C14/I14)</x:f>
+        <x:v>0.23529411764705882</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
@@ -8421,7 +8455,7 @@
     <x:row r="6">
       <x:c r="A6" s="16" t="n">
         <x:f t="shared" ref="A6:F6" si="0">SUM(C11:C20)</x:f>
-        <x:v>138</x:v>
+        <x:v>132</x:v>
       </x:c>
       <x:c r="B6" s="16" t="n">
         <x:f t="shared" si="0"/>
@@ -8805,7 +8839,7 @@
       </x:c>
       <x:c r="C21" s="31" t="n">
         <x:f t="shared" ref="C21:H21" si="1">SUM(C11:C20)</x:f>
-        <x:v>6</x:v>
+        <x:v>132</x:v>
       </x:c>
       <x:c r="D21" s="31" t="n">
         <x:f t="shared" si="1"/>
@@ -11991,69 +12025,101 @@
     </x:row>
     <x:row r="118">
       <x:c r="A118" t="str">
-        <x:v>합계</x:v>
-      </x:c>
-      <x:c r="B118"/>
-      <x:c r="C118"/>
+        <x:v>(주)규람타워렌탈</x:v>
+      </x:c>
+      <x:c r="B118" t="str">
+        <x:v>두산에너빌리티(주)</x:v>
+      </x:c>
+      <x:c r="C118" t="str">
+        <x:v>TERA PROJECT</x:v>
+      </x:c>
       <x:c r="D118" s="536" t="n">
-        <x:f>SUM(D106:D117)</x:f>
-        <x:v>51</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="E118" s="536" t="n">
-        <x:f>SUM(E106:E117)</x:f>
-        <x:v>14</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="F118" s="536" t="n">
-        <x:f>SUM(F106:F117)</x:f>
-        <x:v>23</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="G118" s="536" t="n">
-        <x:f>SUM(G106:G117)</x:f>
-        <x:v>2</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="H118" s="536" t="n">
-        <x:f>SUM(H106:H117)</x:f>
-        <x:v>5</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="I118" s="536" t="n">
-        <x:f>SUM(I106:I117)</x:f>
-        <x:v>7</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="J118" t="str">
-        <x:v>※ 미정 7대 (확인된 최신 10월 집계), 다른 월 기록 유지</x:v>
+        <x:v>2026-10-21 신규 / 남부지부</x:v>
       </x:c>
     </x:row>
     <x:row r="119">
       <x:c r="A119" t="str">
-        <x:v>비율 (총대수=100%)</x:v>
+        <x:v>합계</x:v>
       </x:c>
       <x:c r="B119"/>
       <x:c r="C119"/>
-      <x:c r="D119" s="95" t="n">
-        <x:f>IF($D$118=0,0,D118/$D$118)</x:f>
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E119" s="95" t="n">
-        <x:f>IF($D$118=0,0,E118/$D$118)</x:f>
-        <x:v>0.27450980392156865</x:v>
-      </x:c>
-      <x:c r="F119" s="95" t="n">
-        <x:f>IF($D$118=0,0,F118/$D$118)</x:f>
-        <x:v>0.45098039215686275</x:v>
-      </x:c>
-      <x:c r="G119" s="95" t="n">
-        <x:f>IF($D$118=0,0,G118/$D$118)</x:f>
-        <x:v>0.0392156862745098</x:v>
-      </x:c>
-      <x:c r="H119" s="95" t="n">
-        <x:f>IF($D$118=0,0,H118/$D$118)</x:f>
-        <x:v>0.09803921568627451</x:v>
-      </x:c>
-      <x:c r="I119" s="95" t="n">
-        <x:f>IF($D$118=0,0,I118/$D$118)</x:f>
-        <x:v>0.13725490196078433</x:v>
-      </x:c>
-      <x:c r="J119"/>
+      <x:c r="D119" s="536" t="n">
+        <x:f>SUM(D106:D118)</x:f>
+        <x:v>55</x:v>
+      </x:c>
+      <x:c r="E119" s="536" t="n">
+        <x:f>SUM(E106:E118)</x:f>
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="F119" s="536" t="n">
+        <x:f>SUM(F106:F118)</x:f>
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="G119" s="536" t="n">
+        <x:f>SUM(G106:G118)</x:f>
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="H119" s="536" t="n">
+        <x:f>SUM(H106:H118)</x:f>
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="I119" s="536" t="n">
+        <x:f>SUM(I106:I118)</x:f>
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="J119" t="str">
+        <x:v>※ 미정 9대 (10월 신규 현장 합계), 다른 월 기록 유지</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="120">
+      <x:c r="A120" t="str">
+        <x:v>비율 (총대수=100%)</x:v>
+      </x:c>
+      <x:c r="B120"/>
+      <x:c r="C120"/>
+      <x:c r="D120" s="95" t="n">
+        <x:f>IF($D$119=0,0,D119/$D$119)</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E120" s="95" t="n">
+        <x:f>IF($D$119=0,0,E119/$D$119)</x:f>
+        <x:v>0.2727272727272727</x:v>
+      </x:c>
+      <x:c r="F120" s="95" t="n">
+        <x:f>IF($D$119=0,0,F119/$D$119)</x:f>
+        <x:v>0.43636363636363634</x:v>
+      </x:c>
+      <x:c r="G120" s="95" t="n">
+        <x:f>IF($D$119=0,0,G119/$D$119)</x:f>
+        <x:v>0.03636363636363636</x:v>
+      </x:c>
+      <x:c r="H120" s="95" t="n">
+        <x:f>IF($D$119=0,0,H119/$D$119)</x:f>
+        <x:v>0.09090909090909091</x:v>
+      </x:c>
+      <x:c r="I120" s="95" t="n">
+        <x:f>IF($D$119=0,0,I119/$D$119)</x:f>
+        <x:v>0.16363636363636364</x:v>
+      </x:c>
+      <x:c r="J120"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -13170,6 +13236,6 @@
     <x:mergeCell ref="A50:T50"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R24b884fc15174b5f"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R92719184f9344aee"/>
 </x:worksheet>
 </file>
</xml_diff>